<commit_message>
Update model outputs 2026-06-14 18:52:41
</commit_message>
<xml_diff>
--- a/files/t20i_upcoming_boundary_projections_latest.xlsx
+++ b/files/t20i_upcoming_boundary_projections_latest.xlsx
@@ -12,7 +12,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="63" uniqueCount="63">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="113" uniqueCount="113">
   <si>
     <t xml:space="preserve">Date</t>
   </si>
@@ -62,6 +62,150 @@
     <t xml:space="preserve">Total_Boundaries</t>
   </si>
   <si>
+    <t xml:space="preserve">Toss_Neutral_Total_Runs</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Toss_Neutral_Total_4s</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Toss_Neutral_Total_6s</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Toss_Neutral_Total_Boundaries</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Home_Bats_First_Home_Runs</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Home_Bats_First_Away_Runs</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Home_Bats_First_Total_Runs</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Home_Bats_First_Home_4s</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Home_Bats_First_Away_4s</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Home_Bats_First_Total_4s</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Home_Bats_First_Home_6s</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Home_Bats_First_Away_6s</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Home_Bats_First_Total_6s</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Home_Bats_First_Total_Boundaries</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Home_Bats_First_Chase_Target</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Home_Bats_First_Chase_Balls</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Home_Bats_First_Chase_Compression_Balls</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Home_Bats_First_Chase_Method</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Home_Bats_First_Low_Target_Total_Runs</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Home_Bats_First_Low_Target_Total_4s</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Home_Bats_First_Low_Target_Total_6s</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Home_Bats_First_Low_Target_Total_Boundaries</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Home_Bats_First_Base_Target_Total_Boundaries</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Home_Bats_First_High_Target_Total_Boundaries</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Away_Bats_First_Home_Runs</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Away_Bats_First_Away_Runs</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Away_Bats_First_Total_Runs</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Away_Bats_First_Home_4s</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Away_Bats_First_Away_4s</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Away_Bats_First_Total_4s</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Away_Bats_First_Home_6s</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Away_Bats_First_Away_6s</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Away_Bats_First_Total_6s</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Away_Bats_First_Total_Boundaries</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Away_Bats_First_Chase_Target</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Away_Bats_First_Chase_Balls</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Away_Bats_First_Chase_Compression_Balls</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Away_Bats_First_Chase_Method</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Away_Bats_First_Low_Target_Total_Runs</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Away_Bats_First_Low_Target_Total_4s</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Away_Bats_First_Low_Target_Total_6s</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Away_Bats_First_Low_Target_Total_Boundaries</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Away_Bats_First_Base_Target_Total_Boundaries</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Away_Bats_First_High_Target_Total_Boundaries</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Runs_Order_Sensitivity</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Fours_Order_Sensitivity</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Sixes_Order_Sensitivity</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Boundaries_Order_Sensitivity</t>
+  </si>
+  <si>
     <t xml:space="preserve">Venue_Matched</t>
   </si>
   <si>
@@ -129,6 +273,12 @@
   </si>
   <si>
     <t xml:space="preserve">Sri Lanka</t>
+  </si>
+  <si>
+    <t xml:space="preserve">full_innings</t>
+  </si>
+  <si>
+    <t xml:space="preserve">target_chase_compression</t>
   </si>
   <si>
     <t xml:space="preserve">alias_exact</t>
@@ -551,24 +701,72 @@
     <col min="14" max="14" width="8.87326514724293" hidden="0" customWidth="1"/>
     <col min="15" max="15" width="10.0394458825634" hidden="0" customWidth="1"/>
     <col min="16" max="16" width="19.3688917651267" hidden="0" customWidth="1"/>
-    <col min="17" max="17" width="64.7099987543846" hidden="0" customWidth="1"/>
-    <col min="18" max="18" width="15.8703495591654" hidden="0" customWidth="1"/>
-    <col min="19" max="19" width="18.2027110298063" hidden="0" customWidth="1"/>
-    <col min="20" max="20" width="19.3688917651267" hidden="0" customWidth="1"/>
-    <col min="21" max="21" width="18.2027110298063" hidden="0" customWidth="1"/>
-    <col min="22" max="22" width="21.7012532357675" hidden="0" customWidth="1"/>
-    <col min="23" max="23" width="24.7099995328942" hidden="0" customWidth="1"/>
-    <col min="24" max="24" width="24.7099995328942" hidden="0" customWidth="1"/>
-    <col min="25" max="25" width="18.2027110298063" hidden="0" customWidth="1"/>
-    <col min="26" max="26" width="18.2027110298063" hidden="0" customWidth="1"/>
-    <col min="27" max="27" width="21.7012532357675" hidden="0" customWidth="1"/>
-    <col min="28" max="28" width="21.7012532357675" hidden="0" customWidth="1"/>
-    <col min="29" max="29" width="20.5350725004471" hidden="0" customWidth="1"/>
-    <col min="30" max="30" width="20.5350725004471" hidden="0" customWidth="1"/>
-    <col min="31" max="31" width="11.2056266178838" hidden="0" customWidth="1"/>
-    <col min="32" max="32" width="12.3718073532042" hidden="0" customWidth="1"/>
-    <col min="33" max="33" width="11.2056266178838" hidden="0" customWidth="1"/>
-    <col min="34" max="34" width="87.7099983067416" hidden="0" customWidth="1"/>
+    <col min="17" max="17" width="27.5321569123696" hidden="0" customWidth="1"/>
+    <col min="18" max="18" width="25.1997954417288" hidden="0" customWidth="1"/>
+    <col min="19" max="19" width="25.1997954417288" hidden="0" customWidth="1"/>
+    <col min="20" max="20" width="34.5292413242922" hidden="0" customWidth="1"/>
+    <col min="21" max="21" width="29.8645183830105" hidden="0" customWidth="1"/>
+    <col min="22" max="22" width="29.8645183830105" hidden="0" customWidth="1"/>
+    <col min="23" max="23" width="31.0306991183309" hidden="0" customWidth="1"/>
+    <col min="24" max="24" width="27.5321569123696" hidden="0" customWidth="1"/>
+    <col min="25" max="25" width="27.5321569123696" hidden="0" customWidth="1"/>
+    <col min="26" max="26" width="28.6983376476901" hidden="0" customWidth="1"/>
+    <col min="27" max="27" width="27.5321569123696" hidden="0" customWidth="1"/>
+    <col min="28" max="28" width="27.5321569123696" hidden="0" customWidth="1"/>
+    <col min="29" max="29" width="28.6983376476901" hidden="0" customWidth="1"/>
+    <col min="30" max="30" width="38.0277835302534" hidden="0" customWidth="1"/>
+    <col min="31" max="31" width="33.3630605889717" hidden="0" customWidth="1"/>
+    <col min="32" max="32" width="32.1968798536513" hidden="0" customWidth="1"/>
+    <col min="33" max="33" width="46.1910486774963" hidden="0" customWidth="1"/>
+    <col min="34" max="34" width="33.3630605889717" hidden="0" customWidth="1"/>
+    <col min="35" max="35" width="43.8586872068555" hidden="0" customWidth="1"/>
+    <col min="36" max="36" width="41.5263257362147" hidden="0" customWidth="1"/>
+    <col min="37" max="37" width="41.5263257362147" hidden="0" customWidth="1"/>
+    <col min="38" max="38" width="50.855771618778" hidden="0" customWidth="1"/>
+    <col min="39" max="39" width="52.0219523540984" hidden="0" customWidth="1"/>
+    <col min="40" max="40" width="52.0219523540984" hidden="0" customWidth="1"/>
+    <col min="41" max="41" width="29.8645183830105" hidden="0" customWidth="1"/>
+    <col min="42" max="42" width="29.8645183830105" hidden="0" customWidth="1"/>
+    <col min="43" max="43" width="31.0306991183309" hidden="0" customWidth="1"/>
+    <col min="44" max="44" width="27.5321569123696" hidden="0" customWidth="1"/>
+    <col min="45" max="45" width="27.5321569123696" hidden="0" customWidth="1"/>
+    <col min="46" max="46" width="28.6983376476901" hidden="0" customWidth="1"/>
+    <col min="47" max="47" width="27.5321569123696" hidden="0" customWidth="1"/>
+    <col min="48" max="48" width="27.5321569123696" hidden="0" customWidth="1"/>
+    <col min="49" max="49" width="28.6983376476901" hidden="0" customWidth="1"/>
+    <col min="50" max="50" width="38.0277835302534" hidden="0" customWidth="1"/>
+    <col min="51" max="51" width="33.3630605889717" hidden="0" customWidth="1"/>
+    <col min="52" max="52" width="32.1968798536513" hidden="0" customWidth="1"/>
+    <col min="53" max="53" width="46.1910486774963" hidden="0" customWidth="1"/>
+    <col min="54" max="54" width="33.3630605889717" hidden="0" customWidth="1"/>
+    <col min="55" max="55" width="43.8586872068555" hidden="0" customWidth="1"/>
+    <col min="56" max="56" width="41.5263257362147" hidden="0" customWidth="1"/>
+    <col min="57" max="57" width="41.5263257362147" hidden="0" customWidth="1"/>
+    <col min="58" max="58" width="50.855771618778" hidden="0" customWidth="1"/>
+    <col min="59" max="59" width="52.0219523540984" hidden="0" customWidth="1"/>
+    <col min="60" max="60" width="52.0219523540984" hidden="0" customWidth="1"/>
+    <col min="61" max="61" width="26.3659761770492" hidden="0" customWidth="1"/>
+    <col min="62" max="62" width="27.5321569123696" hidden="0" customWidth="1"/>
+    <col min="63" max="63" width="27.5321569123696" hidden="0" customWidth="1"/>
+    <col min="64" max="64" width="33.3630605889717" hidden="0" customWidth="1"/>
+    <col min="65" max="65" width="64.7099987543846" hidden="0" customWidth="1"/>
+    <col min="66" max="66" width="15.8703495591654" hidden="0" customWidth="1"/>
+    <col min="67" max="67" width="18.2027110298063" hidden="0" customWidth="1"/>
+    <col min="68" max="68" width="19.3688917651267" hidden="0" customWidth="1"/>
+    <col min="69" max="69" width="18.2027110298063" hidden="0" customWidth="1"/>
+    <col min="70" max="70" width="21.7012532357675" hidden="0" customWidth="1"/>
+    <col min="71" max="71" width="24.7099995328942" hidden="0" customWidth="1"/>
+    <col min="72" max="72" width="24.7099995328942" hidden="0" customWidth="1"/>
+    <col min="73" max="73" width="18.2027110298063" hidden="0" customWidth="1"/>
+    <col min="74" max="74" width="18.2027110298063" hidden="0" customWidth="1"/>
+    <col min="75" max="75" width="21.7012532357675" hidden="0" customWidth="1"/>
+    <col min="76" max="76" width="21.7012532357675" hidden="0" customWidth="1"/>
+    <col min="77" max="77" width="20.5350725004471" hidden="0" customWidth="1"/>
+    <col min="78" max="78" width="20.5350725004471" hidden="0" customWidth="1"/>
+    <col min="79" max="79" width="11.2056266178838" hidden="0" customWidth="1"/>
+    <col min="80" max="80" width="12.3718073532042" hidden="0" customWidth="1"/>
+    <col min="81" max="81" width="11.2056266178838" hidden="0" customWidth="1"/>
+    <col min="82" max="82" width="87.7099983067416" hidden="0" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -674,34 +872,178 @@
       <c r="AH1" s="2" t="s">
         <v>33</v>
       </c>
+      <c r="AI1" s="2" t="s">
+        <v>34</v>
+      </c>
+      <c r="AJ1" s="2" t="s">
+        <v>35</v>
+      </c>
+      <c r="AK1" s="2" t="s">
+        <v>36</v>
+      </c>
+      <c r="AL1" s="2" t="s">
+        <v>37</v>
+      </c>
+      <c r="AM1" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="AN1" s="2" t="s">
+        <v>39</v>
+      </c>
+      <c r="AO1" s="2" t="s">
+        <v>40</v>
+      </c>
+      <c r="AP1" s="2" t="s">
+        <v>41</v>
+      </c>
+      <c r="AQ1" s="2" t="s">
+        <v>42</v>
+      </c>
+      <c r="AR1" s="2" t="s">
+        <v>43</v>
+      </c>
+      <c r="AS1" s="2" t="s">
+        <v>44</v>
+      </c>
+      <c r="AT1" s="2" t="s">
+        <v>45</v>
+      </c>
+      <c r="AU1" s="2" t="s">
+        <v>46</v>
+      </c>
+      <c r="AV1" s="2" t="s">
+        <v>47</v>
+      </c>
+      <c r="AW1" s="2" t="s">
+        <v>48</v>
+      </c>
+      <c r="AX1" s="2" t="s">
+        <v>49</v>
+      </c>
+      <c r="AY1" s="2" t="s">
+        <v>50</v>
+      </c>
+      <c r="AZ1" s="2" t="s">
+        <v>51</v>
+      </c>
+      <c r="BA1" s="2" t="s">
+        <v>52</v>
+      </c>
+      <c r="BB1" s="2" t="s">
+        <v>53</v>
+      </c>
+      <c r="BC1" s="2" t="s">
+        <v>54</v>
+      </c>
+      <c r="BD1" s="2" t="s">
+        <v>55</v>
+      </c>
+      <c r="BE1" s="2" t="s">
+        <v>56</v>
+      </c>
+      <c r="BF1" s="2" t="s">
+        <v>57</v>
+      </c>
+      <c r="BG1" s="2" t="s">
+        <v>58</v>
+      </c>
+      <c r="BH1" s="2" t="s">
+        <v>59</v>
+      </c>
+      <c r="BI1" s="2" t="s">
+        <v>60</v>
+      </c>
+      <c r="BJ1" s="2" t="s">
+        <v>61</v>
+      </c>
+      <c r="BK1" s="2" t="s">
+        <v>62</v>
+      </c>
+      <c r="BL1" s="2" t="s">
+        <v>63</v>
+      </c>
+      <c r="BM1" s="2" t="s">
+        <v>64</v>
+      </c>
+      <c r="BN1" s="2" t="s">
+        <v>65</v>
+      </c>
+      <c r="BO1" s="2" t="s">
+        <v>66</v>
+      </c>
+      <c r="BP1" s="2" t="s">
+        <v>67</v>
+      </c>
+      <c r="BQ1" s="2" t="s">
+        <v>68</v>
+      </c>
+      <c r="BR1" s="2" t="s">
+        <v>69</v>
+      </c>
+      <c r="BS1" s="2" t="s">
+        <v>70</v>
+      </c>
+      <c r="BT1" s="2" t="s">
+        <v>71</v>
+      </c>
+      <c r="BU1" s="2" t="s">
+        <v>72</v>
+      </c>
+      <c r="BV1" s="2" t="s">
+        <v>73</v>
+      </c>
+      <c r="BW1" s="2" t="s">
+        <v>74</v>
+      </c>
+      <c r="BX1" s="2" t="s">
+        <v>75</v>
+      </c>
+      <c r="BY1" s="2" t="s">
+        <v>76</v>
+      </c>
+      <c r="BZ1" s="2" t="s">
+        <v>77</v>
+      </c>
+      <c r="CA1" s="2" t="s">
+        <v>78</v>
+      </c>
+      <c r="CB1" s="2" t="s">
+        <v>79</v>
+      </c>
+      <c r="CC1" s="2" t="s">
+        <v>80</v>
+      </c>
+      <c r="CD1" s="2" t="s">
+        <v>81</v>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="1" t="n">
         <v>46187</v>
       </c>
       <c r="B2" t="s">
-        <v>34</v>
+        <v>82</v>
       </c>
       <c r="C2" t="s">
-        <v>35</v>
+        <v>83</v>
       </c>
       <c r="D2" t="s">
-        <v>36</v>
+        <v>84</v>
       </c>
       <c r="E2" t="s">
-        <v>37</v>
+        <v>85</v>
       </c>
       <c r="F2" t="s">
-        <v>38</v>
+        <v>86</v>
       </c>
       <c r="G2" t="n">
-        <v>192</v>
+        <v>188.1</v>
       </c>
       <c r="H2" t="n">
         <v>188.1</v>
       </c>
       <c r="I2" t="n">
-        <v>380.1</v>
+        <v>376.2</v>
       </c>
       <c r="J2" t="n">
         <v>13.2</v>
@@ -713,7 +1055,7 @@
         <v>27.9</v>
       </c>
       <c r="M2" t="n">
-        <v>11.7</v>
+        <v>11.6</v>
       </c>
       <c r="N2" t="n">
         <v>7.9</v>
@@ -722,61 +1064,205 @@
         <v>19.6</v>
       </c>
       <c r="P2" t="n">
-        <v>47.5</v>
-      </c>
-      <c r="Q2" t="s">
-        <v>36</v>
+        <v>47.4</v>
+      </c>
+      <c r="Q2" t="n">
+        <v>376.2</v>
       </c>
       <c r="R2" t="n">
+        <v>27.9</v>
+      </c>
+      <c r="S2" t="n">
+        <v>19.6</v>
+      </c>
+      <c r="T2" t="n">
+        <v>47.4</v>
+      </c>
+      <c r="U2" t="n">
+        <v>193.2</v>
+      </c>
+      <c r="V2" t="n">
+        <v>186.9</v>
+      </c>
+      <c r="W2" t="n">
+        <v>380.2</v>
+      </c>
+      <c r="X2" t="n">
+        <v>12.8</v>
+      </c>
+      <c r="Y2" t="n">
+        <v>15.1</v>
+      </c>
+      <c r="Z2" t="n">
+        <v>28</v>
+      </c>
+      <c r="AA2" t="n">
+        <v>12.1</v>
+      </c>
+      <c r="AB2" t="n">
+        <v>7.6</v>
+      </c>
+      <c r="AC2" t="n">
+        <v>19.7</v>
+      </c>
+      <c r="AD2" t="n">
+        <v>47.7</v>
+      </c>
+      <c r="AE2" t="n">
+        <v>194</v>
+      </c>
+      <c r="AF2" t="n">
+        <v>120</v>
+      </c>
+      <c r="AG2" t="n">
+        <v>0</v>
+      </c>
+      <c r="AH2" t="s">
+        <v>87</v>
+      </c>
+      <c r="AI2" t="n">
+        <v>345.4</v>
+      </c>
+      <c r="AJ2" t="n">
+        <v>25.7</v>
+      </c>
+      <c r="AK2" t="n">
+        <v>17.6</v>
+      </c>
+      <c r="AL2" t="n">
+        <v>43.2</v>
+      </c>
+      <c r="AM2" t="n">
+        <v>47.7</v>
+      </c>
+      <c r="AN2" t="n">
+        <v>52.2</v>
+      </c>
+      <c r="AO2" t="n">
+        <v>182.9</v>
+      </c>
+      <c r="AP2" t="n">
+        <v>189.3</v>
+      </c>
+      <c r="AQ2" t="n">
+        <v>372.2</v>
+      </c>
+      <c r="AR2" t="n">
+        <v>13.5</v>
+      </c>
+      <c r="AS2" t="n">
+        <v>14.3</v>
+      </c>
+      <c r="AT2" t="n">
+        <v>27.8</v>
+      </c>
+      <c r="AU2" t="n">
+        <v>11.2</v>
+      </c>
+      <c r="AV2" t="n">
+        <v>8.2</v>
+      </c>
+      <c r="AW2" t="n">
+        <v>19.4</v>
+      </c>
+      <c r="AX2" t="n">
+        <v>47.1</v>
+      </c>
+      <c r="AY2" t="n">
+        <v>190</v>
+      </c>
+      <c r="AZ2" t="n">
+        <v>119</v>
+      </c>
+      <c r="BA2" t="n">
+        <v>1</v>
+      </c>
+      <c r="BB2" t="s">
+        <v>88</v>
+      </c>
+      <c r="BC2" t="n">
+        <v>314.2</v>
+      </c>
+      <c r="BD2" t="n">
+        <v>24.9</v>
+      </c>
+      <c r="BE2" t="n">
+        <v>17.6</v>
+      </c>
+      <c r="BF2" t="n">
+        <v>42.5</v>
+      </c>
+      <c r="BG2" t="n">
+        <v>47.3</v>
+      </c>
+      <c r="BH2" t="n">
+        <v>51.4</v>
+      </c>
+      <c r="BI2" t="n">
+        <v>8</v>
+      </c>
+      <c r="BJ2" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="BK2" t="n">
+        <v>0.4</v>
+      </c>
+      <c r="BL2" t="n">
+        <v>0.6</v>
+      </c>
+      <c r="BM2" t="s">
+        <v>84</v>
+      </c>
+      <c r="BN2" t="n">
         <v>16</v>
       </c>
-      <c r="S2" t="n">
+      <c r="BO2" t="n">
         <v>1.13</v>
       </c>
-      <c r="T2" t="n">
+      <c r="BP2" t="n">
         <v>1.039</v>
       </c>
-      <c r="U2" t="n">
+      <c r="BQ2" t="n">
         <v>1.35</v>
       </c>
-      <c r="V2" t="s">
-        <v>39</v>
-      </c>
-      <c r="W2" t="s">
-        <v>40</v>
-      </c>
-      <c r="X2" t="s">
-        <v>40</v>
-      </c>
-      <c r="Y2" t="n">
+      <c r="BR2" t="s">
+        <v>89</v>
+      </c>
+      <c r="BS2" t="s">
+        <v>90</v>
+      </c>
+      <c r="BT2" t="s">
+        <v>90</v>
+      </c>
+      <c r="BU2" t="n">
         <v>10</v>
       </c>
-      <c r="Z2" t="n">
+      <c r="BV2" t="n">
         <v>10</v>
       </c>
-      <c r="AA2" t="n">
+      <c r="BW2" t="n">
         <v>1.023</v>
       </c>
-      <c r="AB2" t="n">
+      <c r="BX2" t="n">
         <v>1.041</v>
       </c>
-      <c r="AC2" t="n">
+      <c r="BY2" t="n">
         <v>1.15</v>
       </c>
-      <c r="AD2" t="n">
+      <c r="BZ2" t="n">
         <v>1.007</v>
       </c>
-      <c r="AE2" t="s">
-        <v>41</v>
-      </c>
-      <c r="AF2" t="s">
-        <v>41</v>
-      </c>
-      <c r="AG2" t="s">
-        <v>41</v>
-      </c>
-      <c r="AH2" t="s">
-        <v>42</v>
+      <c r="CA2" t="s">
+        <v>91</v>
+      </c>
+      <c r="CB2" t="s">
+        <v>91</v>
+      </c>
+      <c r="CC2" t="s">
+        <v>91</v>
+      </c>
+      <c r="CD2" t="s">
+        <v>92</v>
       </c>
     </row>
     <row r="3">
@@ -784,28 +1270,28 @@
         <v>46188</v>
       </c>
       <c r="B3" t="s">
-        <v>34</v>
+        <v>82</v>
       </c>
       <c r="C3" t="s">
-        <v>35</v>
+        <v>83</v>
       </c>
       <c r="D3" t="s">
-        <v>36</v>
+        <v>84</v>
       </c>
       <c r="E3" t="s">
-        <v>37</v>
+        <v>85</v>
       </c>
       <c r="F3" t="s">
-        <v>38</v>
+        <v>86</v>
       </c>
       <c r="G3" t="n">
-        <v>192</v>
+        <v>188.1</v>
       </c>
       <c r="H3" t="n">
         <v>188.1</v>
       </c>
       <c r="I3" t="n">
-        <v>380.1</v>
+        <v>376.2</v>
       </c>
       <c r="J3" t="n">
         <v>13.2</v>
@@ -817,7 +1303,7 @@
         <v>27.9</v>
       </c>
       <c r="M3" t="n">
-        <v>11.7</v>
+        <v>11.6</v>
       </c>
       <c r="N3" t="n">
         <v>7.9</v>
@@ -826,61 +1312,205 @@
         <v>19.6</v>
       </c>
       <c r="P3" t="n">
-        <v>47.5</v>
-      </c>
-      <c r="Q3" t="s">
-        <v>36</v>
+        <v>47.4</v>
+      </c>
+      <c r="Q3" t="n">
+        <v>376.2</v>
       </c>
       <c r="R3" t="n">
+        <v>27.9</v>
+      </c>
+      <c r="S3" t="n">
+        <v>19.6</v>
+      </c>
+      <c r="T3" t="n">
+        <v>47.4</v>
+      </c>
+      <c r="U3" t="n">
+        <v>193.2</v>
+      </c>
+      <c r="V3" t="n">
+        <v>186.9</v>
+      </c>
+      <c r="W3" t="n">
+        <v>380.2</v>
+      </c>
+      <c r="X3" t="n">
+        <v>12.8</v>
+      </c>
+      <c r="Y3" t="n">
+        <v>15.1</v>
+      </c>
+      <c r="Z3" t="n">
+        <v>28</v>
+      </c>
+      <c r="AA3" t="n">
+        <v>12.1</v>
+      </c>
+      <c r="AB3" t="n">
+        <v>7.6</v>
+      </c>
+      <c r="AC3" t="n">
+        <v>19.7</v>
+      </c>
+      <c r="AD3" t="n">
+        <v>47.7</v>
+      </c>
+      <c r="AE3" t="n">
+        <v>194</v>
+      </c>
+      <c r="AF3" t="n">
+        <v>120</v>
+      </c>
+      <c r="AG3" t="n">
+        <v>0</v>
+      </c>
+      <c r="AH3" t="s">
+        <v>87</v>
+      </c>
+      <c r="AI3" t="n">
+        <v>345.4</v>
+      </c>
+      <c r="AJ3" t="n">
+        <v>25.7</v>
+      </c>
+      <c r="AK3" t="n">
+        <v>17.6</v>
+      </c>
+      <c r="AL3" t="n">
+        <v>43.2</v>
+      </c>
+      <c r="AM3" t="n">
+        <v>47.7</v>
+      </c>
+      <c r="AN3" t="n">
+        <v>52.2</v>
+      </c>
+      <c r="AO3" t="n">
+        <v>182.9</v>
+      </c>
+      <c r="AP3" t="n">
+        <v>189.3</v>
+      </c>
+      <c r="AQ3" t="n">
+        <v>372.2</v>
+      </c>
+      <c r="AR3" t="n">
+        <v>13.5</v>
+      </c>
+      <c r="AS3" t="n">
+        <v>14.3</v>
+      </c>
+      <c r="AT3" t="n">
+        <v>27.8</v>
+      </c>
+      <c r="AU3" t="n">
+        <v>11.2</v>
+      </c>
+      <c r="AV3" t="n">
+        <v>8.2</v>
+      </c>
+      <c r="AW3" t="n">
+        <v>19.4</v>
+      </c>
+      <c r="AX3" t="n">
+        <v>47.1</v>
+      </c>
+      <c r="AY3" t="n">
+        <v>190</v>
+      </c>
+      <c r="AZ3" t="n">
+        <v>119</v>
+      </c>
+      <c r="BA3" t="n">
+        <v>1</v>
+      </c>
+      <c r="BB3" t="s">
+        <v>88</v>
+      </c>
+      <c r="BC3" t="n">
+        <v>314.2</v>
+      </c>
+      <c r="BD3" t="n">
+        <v>24.9</v>
+      </c>
+      <c r="BE3" t="n">
+        <v>17.6</v>
+      </c>
+      <c r="BF3" t="n">
+        <v>42.5</v>
+      </c>
+      <c r="BG3" t="n">
+        <v>47.3</v>
+      </c>
+      <c r="BH3" t="n">
+        <v>51.4</v>
+      </c>
+      <c r="BI3" t="n">
+        <v>8</v>
+      </c>
+      <c r="BJ3" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="BK3" t="n">
+        <v>0.4</v>
+      </c>
+      <c r="BL3" t="n">
+        <v>0.6</v>
+      </c>
+      <c r="BM3" t="s">
+        <v>84</v>
+      </c>
+      <c r="BN3" t="n">
         <v>16</v>
       </c>
-      <c r="S3" t="n">
+      <c r="BO3" t="n">
         <v>1.13</v>
       </c>
-      <c r="T3" t="n">
+      <c r="BP3" t="n">
         <v>1.039</v>
       </c>
-      <c r="U3" t="n">
+      <c r="BQ3" t="n">
         <v>1.35</v>
       </c>
-      <c r="V3" t="s">
-        <v>39</v>
-      </c>
-      <c r="W3" t="s">
-        <v>40</v>
-      </c>
-      <c r="X3" t="s">
-        <v>40</v>
-      </c>
-      <c r="Y3" t="n">
+      <c r="BR3" t="s">
+        <v>89</v>
+      </c>
+      <c r="BS3" t="s">
+        <v>90</v>
+      </c>
+      <c r="BT3" t="s">
+        <v>90</v>
+      </c>
+      <c r="BU3" t="n">
         <v>10</v>
       </c>
-      <c r="Z3" t="n">
+      <c r="BV3" t="n">
         <v>10</v>
       </c>
-      <c r="AA3" t="n">
+      <c r="BW3" t="n">
         <v>1.023</v>
       </c>
-      <c r="AB3" t="n">
+      <c r="BX3" t="n">
         <v>1.041</v>
       </c>
-      <c r="AC3" t="n">
+      <c r="BY3" t="n">
         <v>1.15</v>
       </c>
-      <c r="AD3" t="n">
+      <c r="BZ3" t="n">
         <v>1.007</v>
       </c>
-      <c r="AE3" t="s">
-        <v>41</v>
-      </c>
-      <c r="AF3" t="s">
-        <v>41</v>
-      </c>
-      <c r="AG3" t="s">
-        <v>41</v>
-      </c>
-      <c r="AH3" t="s">
-        <v>42</v>
+      <c r="CA3" t="s">
+        <v>91</v>
+      </c>
+      <c r="CB3" t="s">
+        <v>91</v>
+      </c>
+      <c r="CC3" t="s">
+        <v>91</v>
+      </c>
+      <c r="CD3" t="s">
+        <v>92</v>
       </c>
     </row>
     <row r="4">
@@ -889,100 +1519,244 @@
       </c>
       <c r="B4"/>
       <c r="C4" t="s">
-        <v>43</v>
+        <v>93</v>
       </c>
       <c r="D4" t="s">
-        <v>44</v>
+        <v>94</v>
       </c>
       <c r="E4" t="s">
-        <v>45</v>
+        <v>95</v>
       </c>
       <c r="F4" t="s">
-        <v>46</v>
+        <v>96</v>
       </c>
       <c r="G4" t="n">
         <v>164.3</v>
       </c>
       <c r="H4" t="n">
-        <v>187</v>
+        <v>181.2</v>
       </c>
       <c r="I4" t="n">
-        <v>351.3</v>
+        <v>345.4</v>
       </c>
       <c r="J4" t="n">
         <v>13.1</v>
       </c>
       <c r="K4" t="n">
-        <v>17.8</v>
+        <v>17.6</v>
       </c>
       <c r="L4" t="n">
-        <v>30.9</v>
+        <v>30.6</v>
       </c>
       <c r="M4" t="n">
         <v>7</v>
       </c>
       <c r="N4" t="n">
-        <v>10.8</v>
+        <v>10.6</v>
       </c>
       <c r="O4" t="n">
+        <v>17.6</v>
+      </c>
+      <c r="P4" t="n">
+        <v>48.3</v>
+      </c>
+      <c r="Q4" t="n">
+        <v>345.4</v>
+      </c>
+      <c r="R4" t="n">
+        <v>30.6</v>
+      </c>
+      <c r="S4" t="n">
+        <v>17.6</v>
+      </c>
+      <c r="T4" t="n">
+        <v>48.3</v>
+      </c>
+      <c r="U4" t="n">
+        <v>165.3</v>
+      </c>
+      <c r="V4" t="n">
+        <v>174.1</v>
+      </c>
+      <c r="W4" t="n">
+        <v>339.4</v>
+      </c>
+      <c r="X4" t="n">
+        <v>12.7</v>
+      </c>
+      <c r="Y4" t="n">
         <v>17.8</v>
       </c>
-      <c r="P4" t="n">
+      <c r="Z4" t="n">
+        <v>30.5</v>
+      </c>
+      <c r="AA4" t="n">
+        <v>7.3</v>
+      </c>
+      <c r="AB4" t="n">
+        <v>10.1</v>
+      </c>
+      <c r="AC4" t="n">
+        <v>17.4</v>
+      </c>
+      <c r="AD4" t="n">
+        <v>47.8</v>
+      </c>
+      <c r="AE4" t="n">
+        <v>166</v>
+      </c>
+      <c r="AF4" t="n">
+        <v>116</v>
+      </c>
+      <c r="AG4" t="n">
+        <v>4</v>
+      </c>
+      <c r="AH4" t="s">
+        <v>88</v>
+      </c>
+      <c r="AI4" t="n">
+        <v>274.6</v>
+      </c>
+      <c r="AJ4" t="n">
+        <v>26.5</v>
+      </c>
+      <c r="AK4" t="n">
+        <v>15.1</v>
+      </c>
+      <c r="AL4" t="n">
+        <v>41.5</v>
+      </c>
+      <c r="AM4" t="n">
         <v>48.7</v>
       </c>
-      <c r="Q4" t="s">
-        <v>47</v>
-      </c>
-      <c r="R4" t="n">
+      <c r="AN4" t="n">
+        <v>52.3</v>
+      </c>
+      <c r="AO4" t="n">
+        <v>163.3</v>
+      </c>
+      <c r="AP4" t="n">
+        <v>188.2</v>
+      </c>
+      <c r="AQ4" t="n">
+        <v>351.4</v>
+      </c>
+      <c r="AR4" t="n">
+        <v>13.4</v>
+      </c>
+      <c r="AS4" t="n">
+        <v>17.3</v>
+      </c>
+      <c r="AT4" t="n">
+        <v>30.8</v>
+      </c>
+      <c r="AU4" t="n">
+        <v>6.8</v>
+      </c>
+      <c r="AV4" t="n">
+        <v>11.1</v>
+      </c>
+      <c r="AW4" t="n">
+        <v>17.9</v>
+      </c>
+      <c r="AX4" t="n">
+        <v>48.7</v>
+      </c>
+      <c r="AY4" t="n">
+        <v>189</v>
+      </c>
+      <c r="AZ4" t="n">
+        <v>120</v>
+      </c>
+      <c r="BA4" t="n">
+        <v>0</v>
+      </c>
+      <c r="BB4" t="s">
+        <v>87</v>
+      </c>
+      <c r="BC4" t="n">
+        <v>317.6</v>
+      </c>
+      <c r="BD4" t="n">
+        <v>27.7</v>
+      </c>
+      <c r="BE4" t="n">
+        <v>15.9</v>
+      </c>
+      <c r="BF4" t="n">
+        <v>43.6</v>
+      </c>
+      <c r="BG4" t="n">
+        <v>48.7</v>
+      </c>
+      <c r="BH4" t="n">
+        <v>53.8</v>
+      </c>
+      <c r="BI4" t="n">
+        <v>12</v>
+      </c>
+      <c r="BJ4" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="BK4" t="n">
+        <v>0.6</v>
+      </c>
+      <c r="BL4" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="BM4" t="s">
+        <v>97</v>
+      </c>
+      <c r="BN4" t="n">
         <v>14</v>
       </c>
-      <c r="S4" t="n">
+      <c r="BO4" t="n">
         <v>1.066</v>
       </c>
-      <c r="T4" t="n">
+      <c r="BP4" t="n">
         <v>1.07</v>
       </c>
-      <c r="U4" t="n">
+      <c r="BQ4" t="n">
         <v>1.136</v>
       </c>
-      <c r="V4" t="s">
-        <v>39</v>
-      </c>
-      <c r="W4" t="s">
-        <v>40</v>
-      </c>
-      <c r="X4" t="s">
-        <v>40</v>
-      </c>
-      <c r="Y4" t="n">
+      <c r="BR4" t="s">
+        <v>89</v>
+      </c>
+      <c r="BS4" t="s">
+        <v>90</v>
+      </c>
+      <c r="BT4" t="s">
+        <v>90</v>
+      </c>
+      <c r="BU4" t="n">
         <v>10</v>
       </c>
-      <c r="Z4" t="n">
+      <c r="BV4" t="n">
         <v>11</v>
       </c>
-      <c r="AA4" t="n">
+      <c r="BW4" t="n">
         <v>1.019</v>
       </c>
-      <c r="AB4" t="n">
+      <c r="BX4" t="n">
         <v>1.15</v>
       </c>
-      <c r="AC4" t="n">
+      <c r="BY4" t="n">
         <v>1.15</v>
       </c>
-      <c r="AD4" t="n">
+      <c r="BZ4" t="n">
         <v>1.15</v>
       </c>
-      <c r="AE4" t="s">
-        <v>41</v>
-      </c>
-      <c r="AF4" t="s">
-        <v>41</v>
-      </c>
-      <c r="AG4" t="s">
-        <v>41</v>
-      </c>
-      <c r="AH4" t="s">
-        <v>48</v>
+      <c r="CA4" t="s">
+        <v>91</v>
+      </c>
+      <c r="CB4" t="s">
+        <v>91</v>
+      </c>
+      <c r="CC4" t="s">
+        <v>91</v>
+      </c>
+      <c r="CD4" t="s">
+        <v>98</v>
       </c>
     </row>
     <row r="5">
@@ -991,100 +1765,244 @@
       </c>
       <c r="B5"/>
       <c r="C5" t="s">
-        <v>43</v>
+        <v>93</v>
       </c>
       <c r="D5" t="s">
-        <v>44</v>
+        <v>94</v>
       </c>
       <c r="E5" t="s">
-        <v>45</v>
+        <v>95</v>
       </c>
       <c r="F5" t="s">
-        <v>46</v>
+        <v>96</v>
       </c>
       <c r="G5" t="n">
         <v>164.3</v>
       </c>
       <c r="H5" t="n">
-        <v>187</v>
+        <v>181.2</v>
       </c>
       <c r="I5" t="n">
-        <v>351.3</v>
+        <v>345.4</v>
       </c>
       <c r="J5" t="n">
         <v>13.1</v>
       </c>
       <c r="K5" t="n">
-        <v>17.8</v>
+        <v>17.6</v>
       </c>
       <c r="L5" t="n">
-        <v>30.9</v>
+        <v>30.6</v>
       </c>
       <c r="M5" t="n">
         <v>7</v>
       </c>
       <c r="N5" t="n">
-        <v>10.8</v>
+        <v>10.6</v>
       </c>
       <c r="O5" t="n">
+        <v>17.6</v>
+      </c>
+      <c r="P5" t="n">
+        <v>48.3</v>
+      </c>
+      <c r="Q5" t="n">
+        <v>345.4</v>
+      </c>
+      <c r="R5" t="n">
+        <v>30.6</v>
+      </c>
+      <c r="S5" t="n">
+        <v>17.6</v>
+      </c>
+      <c r="T5" t="n">
+        <v>48.3</v>
+      </c>
+      <c r="U5" t="n">
+        <v>165.3</v>
+      </c>
+      <c r="V5" t="n">
+        <v>174.1</v>
+      </c>
+      <c r="W5" t="n">
+        <v>339.4</v>
+      </c>
+      <c r="X5" t="n">
+        <v>12.7</v>
+      </c>
+      <c r="Y5" t="n">
         <v>17.8</v>
       </c>
-      <c r="P5" t="n">
+      <c r="Z5" t="n">
+        <v>30.5</v>
+      </c>
+      <c r="AA5" t="n">
+        <v>7.3</v>
+      </c>
+      <c r="AB5" t="n">
+        <v>10.1</v>
+      </c>
+      <c r="AC5" t="n">
+        <v>17.4</v>
+      </c>
+      <c r="AD5" t="n">
+        <v>47.8</v>
+      </c>
+      <c r="AE5" t="n">
+        <v>166</v>
+      </c>
+      <c r="AF5" t="n">
+        <v>116</v>
+      </c>
+      <c r="AG5" t="n">
+        <v>4</v>
+      </c>
+      <c r="AH5" t="s">
+        <v>88</v>
+      </c>
+      <c r="AI5" t="n">
+        <v>274.6</v>
+      </c>
+      <c r="AJ5" t="n">
+        <v>26.5</v>
+      </c>
+      <c r="AK5" t="n">
+        <v>15.1</v>
+      </c>
+      <c r="AL5" t="n">
+        <v>41.5</v>
+      </c>
+      <c r="AM5" t="n">
         <v>48.7</v>
       </c>
-      <c r="Q5" t="s">
-        <v>47</v>
-      </c>
-      <c r="R5" t="n">
+      <c r="AN5" t="n">
+        <v>52.3</v>
+      </c>
+      <c r="AO5" t="n">
+        <v>163.3</v>
+      </c>
+      <c r="AP5" t="n">
+        <v>188.2</v>
+      </c>
+      <c r="AQ5" t="n">
+        <v>351.4</v>
+      </c>
+      <c r="AR5" t="n">
+        <v>13.4</v>
+      </c>
+      <c r="AS5" t="n">
+        <v>17.3</v>
+      </c>
+      <c r="AT5" t="n">
+        <v>30.8</v>
+      </c>
+      <c r="AU5" t="n">
+        <v>6.8</v>
+      </c>
+      <c r="AV5" t="n">
+        <v>11.1</v>
+      </c>
+      <c r="AW5" t="n">
+        <v>17.9</v>
+      </c>
+      <c r="AX5" t="n">
+        <v>48.7</v>
+      </c>
+      <c r="AY5" t="n">
+        <v>189</v>
+      </c>
+      <c r="AZ5" t="n">
+        <v>120</v>
+      </c>
+      <c r="BA5" t="n">
+        <v>0</v>
+      </c>
+      <c r="BB5" t="s">
+        <v>87</v>
+      </c>
+      <c r="BC5" t="n">
+        <v>317.6</v>
+      </c>
+      <c r="BD5" t="n">
+        <v>27.7</v>
+      </c>
+      <c r="BE5" t="n">
+        <v>15.9</v>
+      </c>
+      <c r="BF5" t="n">
+        <v>43.6</v>
+      </c>
+      <c r="BG5" t="n">
+        <v>48.7</v>
+      </c>
+      <c r="BH5" t="n">
+        <v>53.8</v>
+      </c>
+      <c r="BI5" t="n">
+        <v>12</v>
+      </c>
+      <c r="BJ5" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="BK5" t="n">
+        <v>0.6</v>
+      </c>
+      <c r="BL5" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="BM5" t="s">
+        <v>97</v>
+      </c>
+      <c r="BN5" t="n">
         <v>14</v>
       </c>
-      <c r="S5" t="n">
+      <c r="BO5" t="n">
         <v>1.066</v>
       </c>
-      <c r="T5" t="n">
+      <c r="BP5" t="n">
         <v>1.07</v>
       </c>
-      <c r="U5" t="n">
+      <c r="BQ5" t="n">
         <v>1.136</v>
       </c>
-      <c r="V5" t="s">
-        <v>39</v>
-      </c>
-      <c r="W5" t="s">
-        <v>40</v>
-      </c>
-      <c r="X5" t="s">
-        <v>40</v>
-      </c>
-      <c r="Y5" t="n">
+      <c r="BR5" t="s">
+        <v>89</v>
+      </c>
+      <c r="BS5" t="s">
+        <v>90</v>
+      </c>
+      <c r="BT5" t="s">
+        <v>90</v>
+      </c>
+      <c r="BU5" t="n">
         <v>10</v>
       </c>
-      <c r="Z5" t="n">
+      <c r="BV5" t="n">
         <v>11</v>
       </c>
-      <c r="AA5" t="n">
+      <c r="BW5" t="n">
         <v>1.019</v>
       </c>
-      <c r="AB5" t="n">
+      <c r="BX5" t="n">
         <v>1.15</v>
       </c>
-      <c r="AC5" t="n">
+      <c r="BY5" t="n">
         <v>1.15</v>
       </c>
-      <c r="AD5" t="n">
+      <c r="BZ5" t="n">
         <v>1.15</v>
       </c>
-      <c r="AE5" t="s">
-        <v>41</v>
-      </c>
-      <c r="AF5" t="s">
-        <v>41</v>
-      </c>
-      <c r="AG5" t="s">
-        <v>41</v>
-      </c>
-      <c r="AH5" t="s">
-        <v>48</v>
+      <c r="CA5" t="s">
+        <v>91</v>
+      </c>
+      <c r="CB5" t="s">
+        <v>91</v>
+      </c>
+      <c r="CC5" t="s">
+        <v>91</v>
+      </c>
+      <c r="CD5" t="s">
+        <v>98</v>
       </c>
     </row>
     <row r="6">
@@ -1093,100 +2011,244 @@
       </c>
       <c r="B6"/>
       <c r="C6" t="s">
-        <v>43</v>
+        <v>93</v>
       </c>
       <c r="D6" t="s">
-        <v>44</v>
+        <v>94</v>
       </c>
       <c r="E6" t="s">
-        <v>45</v>
+        <v>95</v>
       </c>
       <c r="F6" t="s">
-        <v>46</v>
+        <v>96</v>
       </c>
       <c r="G6" t="n">
         <v>164.3</v>
       </c>
       <c r="H6" t="n">
-        <v>187</v>
+        <v>181.2</v>
       </c>
       <c r="I6" t="n">
-        <v>351.3</v>
+        <v>345.4</v>
       </c>
       <c r="J6" t="n">
         <v>13.1</v>
       </c>
       <c r="K6" t="n">
-        <v>17.8</v>
+        <v>17.6</v>
       </c>
       <c r="L6" t="n">
-        <v>30.9</v>
+        <v>30.6</v>
       </c>
       <c r="M6" t="n">
         <v>7</v>
       </c>
       <c r="N6" t="n">
-        <v>10.8</v>
+        <v>10.6</v>
       </c>
       <c r="O6" t="n">
+        <v>17.6</v>
+      </c>
+      <c r="P6" t="n">
+        <v>48.3</v>
+      </c>
+      <c r="Q6" t="n">
+        <v>345.4</v>
+      </c>
+      <c r="R6" t="n">
+        <v>30.6</v>
+      </c>
+      <c r="S6" t="n">
+        <v>17.6</v>
+      </c>
+      <c r="T6" t="n">
+        <v>48.3</v>
+      </c>
+      <c r="U6" t="n">
+        <v>165.3</v>
+      </c>
+      <c r="V6" t="n">
+        <v>174.1</v>
+      </c>
+      <c r="W6" t="n">
+        <v>339.4</v>
+      </c>
+      <c r="X6" t="n">
+        <v>12.7</v>
+      </c>
+      <c r="Y6" t="n">
         <v>17.8</v>
       </c>
-      <c r="P6" t="n">
+      <c r="Z6" t="n">
+        <v>30.5</v>
+      </c>
+      <c r="AA6" t="n">
+        <v>7.3</v>
+      </c>
+      <c r="AB6" t="n">
+        <v>10.1</v>
+      </c>
+      <c r="AC6" t="n">
+        <v>17.4</v>
+      </c>
+      <c r="AD6" t="n">
+        <v>47.8</v>
+      </c>
+      <c r="AE6" t="n">
+        <v>166</v>
+      </c>
+      <c r="AF6" t="n">
+        <v>116</v>
+      </c>
+      <c r="AG6" t="n">
+        <v>4</v>
+      </c>
+      <c r="AH6" t="s">
+        <v>88</v>
+      </c>
+      <c r="AI6" t="n">
+        <v>274.6</v>
+      </c>
+      <c r="AJ6" t="n">
+        <v>26.5</v>
+      </c>
+      <c r="AK6" t="n">
+        <v>15.1</v>
+      </c>
+      <c r="AL6" t="n">
+        <v>41.5</v>
+      </c>
+      <c r="AM6" t="n">
         <v>48.7</v>
       </c>
-      <c r="Q6" t="s">
-        <v>47</v>
-      </c>
-      <c r="R6" t="n">
+      <c r="AN6" t="n">
+        <v>52.3</v>
+      </c>
+      <c r="AO6" t="n">
+        <v>163.3</v>
+      </c>
+      <c r="AP6" t="n">
+        <v>188.2</v>
+      </c>
+      <c r="AQ6" t="n">
+        <v>351.4</v>
+      </c>
+      <c r="AR6" t="n">
+        <v>13.4</v>
+      </c>
+      <c r="AS6" t="n">
+        <v>17.3</v>
+      </c>
+      <c r="AT6" t="n">
+        <v>30.8</v>
+      </c>
+      <c r="AU6" t="n">
+        <v>6.8</v>
+      </c>
+      <c r="AV6" t="n">
+        <v>11.1</v>
+      </c>
+      <c r="AW6" t="n">
+        <v>17.9</v>
+      </c>
+      <c r="AX6" t="n">
+        <v>48.7</v>
+      </c>
+      <c r="AY6" t="n">
+        <v>189</v>
+      </c>
+      <c r="AZ6" t="n">
+        <v>120</v>
+      </c>
+      <c r="BA6" t="n">
+        <v>0</v>
+      </c>
+      <c r="BB6" t="s">
+        <v>87</v>
+      </c>
+      <c r="BC6" t="n">
+        <v>317.6</v>
+      </c>
+      <c r="BD6" t="n">
+        <v>27.7</v>
+      </c>
+      <c r="BE6" t="n">
+        <v>15.9</v>
+      </c>
+      <c r="BF6" t="n">
+        <v>43.6</v>
+      </c>
+      <c r="BG6" t="n">
+        <v>48.7</v>
+      </c>
+      <c r="BH6" t="n">
+        <v>53.8</v>
+      </c>
+      <c r="BI6" t="n">
+        <v>12</v>
+      </c>
+      <c r="BJ6" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="BK6" t="n">
+        <v>0.6</v>
+      </c>
+      <c r="BL6" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="BM6" t="s">
+        <v>97</v>
+      </c>
+      <c r="BN6" t="n">
         <v>14</v>
       </c>
-      <c r="S6" t="n">
+      <c r="BO6" t="n">
         <v>1.066</v>
       </c>
-      <c r="T6" t="n">
+      <c r="BP6" t="n">
         <v>1.07</v>
       </c>
-      <c r="U6" t="n">
+      <c r="BQ6" t="n">
         <v>1.136</v>
       </c>
-      <c r="V6" t="s">
-        <v>39</v>
-      </c>
-      <c r="W6" t="s">
-        <v>40</v>
-      </c>
-      <c r="X6" t="s">
-        <v>40</v>
-      </c>
-      <c r="Y6" t="n">
+      <c r="BR6" t="s">
+        <v>89</v>
+      </c>
+      <c r="BS6" t="s">
+        <v>90</v>
+      </c>
+      <c r="BT6" t="s">
+        <v>90</v>
+      </c>
+      <c r="BU6" t="n">
         <v>10</v>
       </c>
-      <c r="Z6" t="n">
+      <c r="BV6" t="n">
         <v>11</v>
       </c>
-      <c r="AA6" t="n">
+      <c r="BW6" t="n">
         <v>1.019</v>
       </c>
-      <c r="AB6" t="n">
+      <c r="BX6" t="n">
         <v>1.15</v>
       </c>
-      <c r="AC6" t="n">
+      <c r="BY6" t="n">
         <v>1.15</v>
       </c>
-      <c r="AD6" t="n">
+      <c r="BZ6" t="n">
         <v>1.15</v>
       </c>
-      <c r="AE6" t="s">
-        <v>41</v>
-      </c>
-      <c r="AF6" t="s">
-        <v>41</v>
-      </c>
-      <c r="AG6" t="s">
-        <v>41</v>
-      </c>
-      <c r="AH6" t="s">
-        <v>48</v>
+      <c r="CA6" t="s">
+        <v>91</v>
+      </c>
+      <c r="CB6" t="s">
+        <v>91</v>
+      </c>
+      <c r="CC6" t="s">
+        <v>91</v>
+      </c>
+      <c r="CD6" t="s">
+        <v>98</v>
       </c>
     </row>
     <row r="7">
@@ -1195,100 +2257,244 @@
       </c>
       <c r="B7"/>
       <c r="C7" t="s">
-        <v>49</v>
+        <v>99</v>
       </c>
       <c r="D7" t="s">
-        <v>50</v>
+        <v>100</v>
       </c>
       <c r="E7" t="s">
-        <v>51</v>
+        <v>101</v>
       </c>
       <c r="F7" t="s">
-        <v>52</v>
+        <v>102</v>
       </c>
       <c r="G7" t="n">
         <v>161.5</v>
       </c>
       <c r="H7" t="n">
-        <v>208.2</v>
+        <v>189.2</v>
       </c>
       <c r="I7" t="n">
-        <v>369.7</v>
+        <v>350.7</v>
       </c>
       <c r="J7" t="n">
         <v>16.1</v>
       </c>
       <c r="K7" t="n">
-        <v>21.5</v>
+        <v>20.8</v>
       </c>
       <c r="L7" t="n">
-        <v>37.5</v>
+        <v>36.8</v>
       </c>
       <c r="M7" t="n">
         <v>6.2</v>
       </c>
       <c r="N7" t="n">
-        <v>10.5</v>
+        <v>10.2</v>
       </c>
       <c r="O7" t="n">
-        <v>16.8</v>
+        <v>16.4</v>
       </c>
       <c r="P7" t="n">
+        <v>53.3</v>
+      </c>
+      <c r="Q7" t="n">
+        <v>350.7</v>
+      </c>
+      <c r="R7" t="n">
+        <v>36.8</v>
+      </c>
+      <c r="S7" t="n">
+        <v>16.4</v>
+      </c>
+      <c r="T7" t="n">
+        <v>53.3</v>
+      </c>
+      <c r="U7" t="n">
+        <v>162.5</v>
+      </c>
+      <c r="V7" t="n">
+        <v>169</v>
+      </c>
+      <c r="W7" t="n">
+        <v>331.5</v>
+      </c>
+      <c r="X7" t="n">
+        <v>15.6</v>
+      </c>
+      <c r="Y7" t="n">
+        <v>20.7</v>
+      </c>
+      <c r="Z7" t="n">
+        <v>36.3</v>
+      </c>
+      <c r="AA7" t="n">
+        <v>6.4</v>
+      </c>
+      <c r="AB7" t="n">
+        <v>9.5</v>
+      </c>
+      <c r="AC7" t="n">
+        <v>16</v>
+      </c>
+      <c r="AD7" t="n">
+        <v>52.2</v>
+      </c>
+      <c r="AE7" t="n">
+        <v>163</v>
+      </c>
+      <c r="AF7" t="n">
+        <v>112</v>
+      </c>
+      <c r="AG7" t="n">
+        <v>8</v>
+      </c>
+      <c r="AH7" t="s">
+        <v>88</v>
+      </c>
+      <c r="AI7" t="n">
+        <v>270.3</v>
+      </c>
+      <c r="AJ7" t="n">
+        <v>30.7</v>
+      </c>
+      <c r="AK7" t="n">
+        <v>13.5</v>
+      </c>
+      <c r="AL7" t="n">
+        <v>44.2</v>
+      </c>
+      <c r="AM7" t="n">
+        <v>53.2</v>
+      </c>
+      <c r="AN7" t="n">
+        <v>58.3</v>
+      </c>
+      <c r="AO7" t="n">
+        <v>160.5</v>
+      </c>
+      <c r="AP7" t="n">
+        <v>209.5</v>
+      </c>
+      <c r="AQ7" t="n">
+        <v>370</v>
+      </c>
+      <c r="AR7" t="n">
+        <v>16.5</v>
+      </c>
+      <c r="AS7" t="n">
+        <v>20.9</v>
+      </c>
+      <c r="AT7" t="n">
+        <v>37.4</v>
+      </c>
+      <c r="AU7" t="n">
+        <v>6</v>
+      </c>
+      <c r="AV7" t="n">
+        <v>10.9</v>
+      </c>
+      <c r="AW7" t="n">
+        <v>16.9</v>
+      </c>
+      <c r="AX7" t="n">
         <v>54.3</v>
       </c>
-      <c r="Q7" t="s">
-        <v>53</v>
-      </c>
-      <c r="R7" t="n">
+      <c r="AY7" t="n">
+        <v>210</v>
+      </c>
+      <c r="AZ7" t="n">
+        <v>120</v>
+      </c>
+      <c r="BA7" t="n">
+        <v>0</v>
+      </c>
+      <c r="BB7" t="s">
+        <v>87</v>
+      </c>
+      <c r="BC7" t="n">
+        <v>335</v>
+      </c>
+      <c r="BD7" t="n">
+        <v>33.9</v>
+      </c>
+      <c r="BE7" t="n">
+        <v>15.1</v>
+      </c>
+      <c r="BF7" t="n">
+        <v>49</v>
+      </c>
+      <c r="BG7" t="n">
+        <v>54.3</v>
+      </c>
+      <c r="BH7" t="n">
+        <v>59.6</v>
+      </c>
+      <c r="BI7" t="n">
+        <v>38.5</v>
+      </c>
+      <c r="BJ7" t="n">
+        <v>1.1</v>
+      </c>
+      <c r="BK7" t="n">
+        <v>1</v>
+      </c>
+      <c r="BL7" t="n">
+        <v>2.1</v>
+      </c>
+      <c r="BM7" t="s">
+        <v>103</v>
+      </c>
+      <c r="BN7" t="n">
         <v>10</v>
       </c>
-      <c r="S7" t="n">
+      <c r="BO7" t="n">
         <v>1.054</v>
       </c>
-      <c r="T7" t="n">
+      <c r="BP7" t="n">
         <v>1.114</v>
       </c>
-      <c r="U7" t="n">
+      <c r="BQ7" t="n">
         <v>1.011</v>
       </c>
-      <c r="V7" t="s">
-        <v>39</v>
-      </c>
-      <c r="W7" t="s">
-        <v>40</v>
-      </c>
-      <c r="X7" t="s">
-        <v>40</v>
-      </c>
-      <c r="Y7" t="n">
+      <c r="BR7" t="s">
+        <v>89</v>
+      </c>
+      <c r="BS7" t="s">
+        <v>90</v>
+      </c>
+      <c r="BT7" t="s">
+        <v>90</v>
+      </c>
+      <c r="BU7" t="n">
         <v>10</v>
       </c>
-      <c r="Z7" t="n">
+      <c r="BV7" t="n">
         <v>9</v>
       </c>
-      <c r="AA7" t="n">
+      <c r="BW7" t="n">
         <v>1.1</v>
       </c>
-      <c r="AB7" t="n">
+      <c r="BX7" t="n">
         <v>1.15</v>
       </c>
-      <c r="AC7" t="n">
+      <c r="BY7" t="n">
         <v>1.137</v>
       </c>
-      <c r="AD7" t="n">
+      <c r="BZ7" t="n">
         <v>1.15</v>
       </c>
-      <c r="AE7" t="s">
-        <v>41</v>
-      </c>
-      <c r="AF7" t="s">
-        <v>41</v>
-      </c>
-      <c r="AG7" t="s">
-        <v>41</v>
-      </c>
-      <c r="AH7" t="s">
-        <v>54</v>
+      <c r="CA7" t="s">
+        <v>91</v>
+      </c>
+      <c r="CB7" t="s">
+        <v>91</v>
+      </c>
+      <c r="CC7" t="s">
+        <v>91</v>
+      </c>
+      <c r="CD7" t="s">
+        <v>104</v>
       </c>
     </row>
     <row r="8">
@@ -1297,100 +2503,244 @@
       </c>
       <c r="B8"/>
       <c r="C8" t="s">
-        <v>49</v>
+        <v>99</v>
       </c>
       <c r="D8" t="s">
-        <v>50</v>
+        <v>100</v>
       </c>
       <c r="E8" t="s">
-        <v>51</v>
+        <v>101</v>
       </c>
       <c r="F8" t="s">
-        <v>52</v>
+        <v>102</v>
       </c>
       <c r="G8" t="n">
         <v>161.5</v>
       </c>
       <c r="H8" t="n">
-        <v>208.2</v>
+        <v>189.2</v>
       </c>
       <c r="I8" t="n">
-        <v>369.7</v>
+        <v>350.7</v>
       </c>
       <c r="J8" t="n">
         <v>16.1</v>
       </c>
       <c r="K8" t="n">
-        <v>21.5</v>
+        <v>20.8</v>
       </c>
       <c r="L8" t="n">
-        <v>37.5</v>
+        <v>36.8</v>
       </c>
       <c r="M8" t="n">
         <v>6.2</v>
       </c>
       <c r="N8" t="n">
-        <v>10.5</v>
+        <v>10.2</v>
       </c>
       <c r="O8" t="n">
-        <v>16.8</v>
+        <v>16.4</v>
       </c>
       <c r="P8" t="n">
+        <v>53.3</v>
+      </c>
+      <c r="Q8" t="n">
+        <v>350.7</v>
+      </c>
+      <c r="R8" t="n">
+        <v>36.8</v>
+      </c>
+      <c r="S8" t="n">
+        <v>16.4</v>
+      </c>
+      <c r="T8" t="n">
+        <v>53.3</v>
+      </c>
+      <c r="U8" t="n">
+        <v>162.5</v>
+      </c>
+      <c r="V8" t="n">
+        <v>169</v>
+      </c>
+      <c r="W8" t="n">
+        <v>331.5</v>
+      </c>
+      <c r="X8" t="n">
+        <v>15.6</v>
+      </c>
+      <c r="Y8" t="n">
+        <v>20.7</v>
+      </c>
+      <c r="Z8" t="n">
+        <v>36.3</v>
+      </c>
+      <c r="AA8" t="n">
+        <v>6.4</v>
+      </c>
+      <c r="AB8" t="n">
+        <v>9.5</v>
+      </c>
+      <c r="AC8" t="n">
+        <v>16</v>
+      </c>
+      <c r="AD8" t="n">
+        <v>52.2</v>
+      </c>
+      <c r="AE8" t="n">
+        <v>163</v>
+      </c>
+      <c r="AF8" t="n">
+        <v>112</v>
+      </c>
+      <c r="AG8" t="n">
+        <v>8</v>
+      </c>
+      <c r="AH8" t="s">
+        <v>88</v>
+      </c>
+      <c r="AI8" t="n">
+        <v>270.3</v>
+      </c>
+      <c r="AJ8" t="n">
+        <v>30.7</v>
+      </c>
+      <c r="AK8" t="n">
+        <v>13.5</v>
+      </c>
+      <c r="AL8" t="n">
+        <v>44.2</v>
+      </c>
+      <c r="AM8" t="n">
+        <v>53.2</v>
+      </c>
+      <c r="AN8" t="n">
+        <v>58.3</v>
+      </c>
+      <c r="AO8" t="n">
+        <v>160.5</v>
+      </c>
+      <c r="AP8" t="n">
+        <v>209.5</v>
+      </c>
+      <c r="AQ8" t="n">
+        <v>370</v>
+      </c>
+      <c r="AR8" t="n">
+        <v>16.5</v>
+      </c>
+      <c r="AS8" t="n">
+        <v>20.9</v>
+      </c>
+      <c r="AT8" t="n">
+        <v>37.4</v>
+      </c>
+      <c r="AU8" t="n">
+        <v>6</v>
+      </c>
+      <c r="AV8" t="n">
+        <v>10.9</v>
+      </c>
+      <c r="AW8" t="n">
+        <v>16.9</v>
+      </c>
+      <c r="AX8" t="n">
         <v>54.3</v>
       </c>
-      <c r="Q8" t="s">
-        <v>53</v>
-      </c>
-      <c r="R8" t="n">
+      <c r="AY8" t="n">
+        <v>210</v>
+      </c>
+      <c r="AZ8" t="n">
+        <v>120</v>
+      </c>
+      <c r="BA8" t="n">
+        <v>0</v>
+      </c>
+      <c r="BB8" t="s">
+        <v>87</v>
+      </c>
+      <c r="BC8" t="n">
+        <v>335</v>
+      </c>
+      <c r="BD8" t="n">
+        <v>33.9</v>
+      </c>
+      <c r="BE8" t="n">
+        <v>15.1</v>
+      </c>
+      <c r="BF8" t="n">
+        <v>49</v>
+      </c>
+      <c r="BG8" t="n">
+        <v>54.3</v>
+      </c>
+      <c r="BH8" t="n">
+        <v>59.6</v>
+      </c>
+      <c r="BI8" t="n">
+        <v>38.5</v>
+      </c>
+      <c r="BJ8" t="n">
+        <v>1.1</v>
+      </c>
+      <c r="BK8" t="n">
+        <v>1</v>
+      </c>
+      <c r="BL8" t="n">
+        <v>2.1</v>
+      </c>
+      <c r="BM8" t="s">
+        <v>103</v>
+      </c>
+      <c r="BN8" t="n">
         <v>10</v>
       </c>
-      <c r="S8" t="n">
+      <c r="BO8" t="n">
         <v>1.054</v>
       </c>
-      <c r="T8" t="n">
+      <c r="BP8" t="n">
         <v>1.114</v>
       </c>
-      <c r="U8" t="n">
+      <c r="BQ8" t="n">
         <v>1.011</v>
       </c>
-      <c r="V8" t="s">
-        <v>39</v>
-      </c>
-      <c r="W8" t="s">
-        <v>40</v>
-      </c>
-      <c r="X8" t="s">
-        <v>40</v>
-      </c>
-      <c r="Y8" t="n">
+      <c r="BR8" t="s">
+        <v>89</v>
+      </c>
+      <c r="BS8" t="s">
+        <v>90</v>
+      </c>
+      <c r="BT8" t="s">
+        <v>90</v>
+      </c>
+      <c r="BU8" t="n">
         <v>10</v>
       </c>
-      <c r="Z8" t="n">
+      <c r="BV8" t="n">
         <v>9</v>
       </c>
-      <c r="AA8" t="n">
+      <c r="BW8" t="n">
         <v>1.1</v>
       </c>
-      <c r="AB8" t="n">
+      <c r="BX8" t="n">
         <v>1.15</v>
       </c>
-      <c r="AC8" t="n">
+      <c r="BY8" t="n">
         <v>1.137</v>
       </c>
-      <c r="AD8" t="n">
+      <c r="BZ8" t="n">
         <v>1.15</v>
       </c>
-      <c r="AE8" t="s">
-        <v>41</v>
-      </c>
-      <c r="AF8" t="s">
-        <v>41</v>
-      </c>
-      <c r="AG8" t="s">
-        <v>41</v>
-      </c>
-      <c r="AH8" t="s">
-        <v>54</v>
+      <c r="CA8" t="s">
+        <v>91</v>
+      </c>
+      <c r="CB8" t="s">
+        <v>91</v>
+      </c>
+      <c r="CC8" t="s">
+        <v>91</v>
+      </c>
+      <c r="CD8" t="s">
+        <v>104</v>
       </c>
     </row>
     <row r="9">
@@ -1399,100 +2749,244 @@
       </c>
       <c r="B9"/>
       <c r="C9" t="s">
-        <v>55</v>
+        <v>105</v>
       </c>
       <c r="D9" t="s">
-        <v>56</v>
+        <v>106</v>
       </c>
       <c r="E9" t="s">
-        <v>57</v>
+        <v>107</v>
       </c>
       <c r="F9" t="s">
-        <v>52</v>
+        <v>102</v>
       </c>
       <c r="G9" t="n">
         <v>185.4</v>
       </c>
       <c r="H9" t="n">
-        <v>200.1</v>
+        <v>194.8</v>
       </c>
       <c r="I9" t="n">
-        <v>385.6</v>
+        <v>380.2</v>
       </c>
       <c r="J9" t="n">
         <v>17.4</v>
       </c>
       <c r="K9" t="n">
-        <v>18.8</v>
+        <v>18.7</v>
       </c>
       <c r="L9" t="n">
-        <v>36.2</v>
+        <v>36</v>
       </c>
       <c r="M9" t="n">
         <v>10.2</v>
       </c>
       <c r="N9" t="n">
-        <v>12.9</v>
+        <v>12.8</v>
       </c>
       <c r="O9" t="n">
-        <v>23</v>
+        <v>22.9</v>
       </c>
       <c r="P9" t="n">
+        <v>58.9</v>
+      </c>
+      <c r="Q9" t="n">
+        <v>380.2</v>
+      </c>
+      <c r="R9" t="n">
+        <v>36</v>
+      </c>
+      <c r="S9" t="n">
+        <v>22.9</v>
+      </c>
+      <c r="T9" t="n">
+        <v>58.9</v>
+      </c>
+      <c r="U9" t="n">
+        <v>186.6</v>
+      </c>
+      <c r="V9" t="n">
+        <v>188.2</v>
+      </c>
+      <c r="W9" t="n">
+        <v>374.8</v>
+      </c>
+      <c r="X9" t="n">
+        <v>16.9</v>
+      </c>
+      <c r="Y9" t="n">
+        <v>19</v>
+      </c>
+      <c r="Z9" t="n">
+        <v>35.9</v>
+      </c>
+      <c r="AA9" t="n">
+        <v>10.5</v>
+      </c>
+      <c r="AB9" t="n">
+        <v>12.2</v>
+      </c>
+      <c r="AC9" t="n">
+        <v>22.7</v>
+      </c>
+      <c r="AD9" t="n">
+        <v>58.6</v>
+      </c>
+      <c r="AE9" t="n">
+        <v>187</v>
+      </c>
+      <c r="AF9" t="n">
+        <v>118</v>
+      </c>
+      <c r="AG9" t="n">
+        <v>2</v>
+      </c>
+      <c r="AH9" t="s">
+        <v>88</v>
+      </c>
+      <c r="AI9" t="n">
+        <v>309</v>
+      </c>
+      <c r="AJ9" t="n">
+        <v>31.9</v>
+      </c>
+      <c r="AK9" t="n">
+        <v>20.2</v>
+      </c>
+      <c r="AL9" t="n">
+        <v>52.1</v>
+      </c>
+      <c r="AM9" t="n">
         <v>59.2</v>
       </c>
-      <c r="Q9" t="s">
-        <v>56</v>
-      </c>
-      <c r="R9" t="n">
+      <c r="AN9" t="n">
+        <v>64.1</v>
+      </c>
+      <c r="AO9" t="n">
+        <v>184.3</v>
+      </c>
+      <c r="AP9" t="n">
+        <v>201.4</v>
+      </c>
+      <c r="AQ9" t="n">
+        <v>385.7</v>
+      </c>
+      <c r="AR9" t="n">
+        <v>17.9</v>
+      </c>
+      <c r="AS9" t="n">
+        <v>18.3</v>
+      </c>
+      <c r="AT9" t="n">
+        <v>36.2</v>
+      </c>
+      <c r="AU9" t="n">
+        <v>9.8</v>
+      </c>
+      <c r="AV9" t="n">
+        <v>13.3</v>
+      </c>
+      <c r="AW9" t="n">
+        <v>23.1</v>
+      </c>
+      <c r="AX9" t="n">
+        <v>59.3</v>
+      </c>
+      <c r="AY9" t="n">
+        <v>202</v>
+      </c>
+      <c r="AZ9" t="n">
+        <v>120</v>
+      </c>
+      <c r="BA9" t="n">
+        <v>0</v>
+      </c>
+      <c r="BB9" t="s">
+        <v>87</v>
+      </c>
+      <c r="BC9" t="n">
+        <v>350.7</v>
+      </c>
+      <c r="BD9" t="n">
+        <v>33</v>
+      </c>
+      <c r="BE9" t="n">
+        <v>20.8</v>
+      </c>
+      <c r="BF9" t="n">
+        <v>53.8</v>
+      </c>
+      <c r="BG9" t="n">
+        <v>59.3</v>
+      </c>
+      <c r="BH9" t="n">
+        <v>64.8</v>
+      </c>
+      <c r="BI9" t="n">
+        <v>10.9</v>
+      </c>
+      <c r="BJ9" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="BK9" t="n">
+        <v>0.4</v>
+      </c>
+      <c r="BL9" t="n">
+        <v>0.6</v>
+      </c>
+      <c r="BM9" t="s">
+        <v>106</v>
+      </c>
+      <c r="BN9" t="n">
         <v>4</v>
       </c>
-      <c r="S9" t="n">
+      <c r="BO9" t="n">
         <v>1.036</v>
       </c>
-      <c r="T9" t="n">
+      <c r="BP9" t="n">
         <v>1.016</v>
       </c>
-      <c r="U9" t="n">
+      <c r="BQ9" t="n">
         <v>1.077</v>
       </c>
-      <c r="V9" t="s">
-        <v>39</v>
-      </c>
-      <c r="W9" t="s">
-        <v>40</v>
-      </c>
-      <c r="X9" t="s">
-        <v>40</v>
-      </c>
-      <c r="Y9" t="n">
+      <c r="BR9" t="s">
+        <v>89</v>
+      </c>
+      <c r="BS9" t="s">
+        <v>90</v>
+      </c>
+      <c r="BT9" t="s">
+        <v>90</v>
+      </c>
+      <c r="BU9" t="n">
         <v>11</v>
       </c>
-      <c r="Z9" t="n">
+      <c r="BV9" t="n">
         <v>9</v>
       </c>
-      <c r="AA9" t="n">
+      <c r="BW9" t="n">
         <v>1.15</v>
       </c>
-      <c r="AB9" t="n">
+      <c r="BX9" t="n">
         <v>1.15</v>
       </c>
-      <c r="AC9" t="n">
+      <c r="BY9" t="n">
         <v>1.15</v>
       </c>
-      <c r="AD9" t="n">
+      <c r="BZ9" t="n">
         <v>1.15</v>
       </c>
-      <c r="AE9" t="s">
-        <v>41</v>
-      </c>
-      <c r="AF9" t="s">
-        <v>41</v>
-      </c>
-      <c r="AG9" t="s">
-        <v>41</v>
-      </c>
-      <c r="AH9" t="s">
-        <v>42</v>
+      <c r="CA9" t="s">
+        <v>91</v>
+      </c>
+      <c r="CB9" t="s">
+        <v>91</v>
+      </c>
+      <c r="CC9" t="s">
+        <v>91</v>
+      </c>
+      <c r="CD9" t="s">
+        <v>92</v>
       </c>
     </row>
     <row r="10">
@@ -1501,100 +2995,244 @@
       </c>
       <c r="B10"/>
       <c r="C10" t="s">
-        <v>55</v>
+        <v>105</v>
       </c>
       <c r="D10" t="s">
-        <v>58</v>
+        <v>108</v>
       </c>
       <c r="E10" t="s">
-        <v>57</v>
+        <v>107</v>
       </c>
       <c r="F10" t="s">
-        <v>52</v>
+        <v>102</v>
       </c>
       <c r="G10" t="n">
         <v>193.4</v>
       </c>
       <c r="H10" t="n">
-        <v>208.8</v>
+        <v>203.2</v>
       </c>
       <c r="I10" t="n">
-        <v>402.2</v>
+        <v>396.6</v>
       </c>
       <c r="J10" t="n">
         <v>19.3</v>
       </c>
       <c r="K10" t="n">
-        <v>20.9</v>
+        <v>20.8</v>
       </c>
       <c r="L10" t="n">
-        <v>40.2</v>
+        <v>40.1</v>
       </c>
       <c r="M10" t="n">
         <v>11.3</v>
       </c>
       <c r="N10" t="n">
-        <v>14.3</v>
+        <v>14.2</v>
       </c>
       <c r="O10" t="n">
-        <v>25.6</v>
+        <v>25.5</v>
       </c>
       <c r="P10" t="n">
-        <v>65.8</v>
-      </c>
-      <c r="Q10" t="s">
-        <v>58</v>
+        <v>65.6</v>
+      </c>
+      <c r="Q10" t="n">
+        <v>396.6</v>
       </c>
       <c r="R10" t="n">
+        <v>40.1</v>
+      </c>
+      <c r="S10" t="n">
+        <v>25.5</v>
+      </c>
+      <c r="T10" t="n">
+        <v>65.6</v>
+      </c>
+      <c r="U10" t="n">
+        <v>194.6</v>
+      </c>
+      <c r="V10" t="n">
+        <v>196.4</v>
+      </c>
+      <c r="W10" t="n">
+        <v>391</v>
+      </c>
+      <c r="X10" t="n">
+        <v>18.7</v>
+      </c>
+      <c r="Y10" t="n">
+        <v>21.2</v>
+      </c>
+      <c r="Z10" t="n">
+        <v>40</v>
+      </c>
+      <c r="AA10" t="n">
+        <v>11.7</v>
+      </c>
+      <c r="AB10" t="n">
+        <v>13.6</v>
+      </c>
+      <c r="AC10" t="n">
+        <v>25.3</v>
+      </c>
+      <c r="AD10" t="n">
+        <v>65.3</v>
+      </c>
+      <c r="AE10" t="n">
+        <v>195</v>
+      </c>
+      <c r="AF10" t="n">
+        <v>118</v>
+      </c>
+      <c r="AG10" t="n">
+        <v>2</v>
+      </c>
+      <c r="AH10" t="s">
+        <v>88</v>
+      </c>
+      <c r="AI10" t="n">
+        <v>322.6</v>
+      </c>
+      <c r="AJ10" t="n">
+        <v>35.8</v>
+      </c>
+      <c r="AK10" t="n">
+        <v>22.7</v>
+      </c>
+      <c r="AL10" t="n">
+        <v>58.5</v>
+      </c>
+      <c r="AM10" t="n">
+        <v>65.7</v>
+      </c>
+      <c r="AN10" t="n">
+        <v>71.2</v>
+      </c>
+      <c r="AO10" t="n">
+        <v>192.2</v>
+      </c>
+      <c r="AP10" t="n">
+        <v>210.1</v>
+      </c>
+      <c r="AQ10" t="n">
+        <v>402.3</v>
+      </c>
+      <c r="AR10" t="n">
+        <v>19.9</v>
+      </c>
+      <c r="AS10" t="n">
+        <v>20.3</v>
+      </c>
+      <c r="AT10" t="n">
+        <v>40.2</v>
+      </c>
+      <c r="AU10" t="n">
+        <v>10.9</v>
+      </c>
+      <c r="AV10" t="n">
+        <v>14.8</v>
+      </c>
+      <c r="AW10" t="n">
+        <v>25.7</v>
+      </c>
+      <c r="AX10" t="n">
+        <v>65.9</v>
+      </c>
+      <c r="AY10" t="n">
+        <v>211</v>
+      </c>
+      <c r="AZ10" t="n">
+        <v>120</v>
+      </c>
+      <c r="BA10" t="n">
+        <v>0</v>
+      </c>
+      <c r="BB10" t="s">
+        <v>87</v>
+      </c>
+      <c r="BC10" t="n">
+        <v>367.3</v>
+      </c>
+      <c r="BD10" t="n">
+        <v>36.8</v>
+      </c>
+      <c r="BE10" t="n">
+        <v>23.2</v>
+      </c>
+      <c r="BF10" t="n">
+        <v>60</v>
+      </c>
+      <c r="BG10" t="n">
+        <v>65.9</v>
+      </c>
+      <c r="BH10" t="n">
+        <v>71.7</v>
+      </c>
+      <c r="BI10" t="n">
+        <v>11.3</v>
+      </c>
+      <c r="BJ10" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="BK10" t="n">
+        <v>0.4</v>
+      </c>
+      <c r="BL10" t="n">
+        <v>0.6</v>
+      </c>
+      <c r="BM10" t="s">
+        <v>108</v>
+      </c>
+      <c r="BN10" t="n">
         <v>6</v>
       </c>
-      <c r="S10" t="n">
+      <c r="BO10" t="n">
         <v>1.081</v>
       </c>
-      <c r="T10" t="n">
+      <c r="BP10" t="n">
         <v>1.128</v>
       </c>
-      <c r="U10" t="n">
+      <c r="BQ10" t="n">
         <v>1.199</v>
       </c>
-      <c r="V10" t="s">
-        <v>39</v>
-      </c>
-      <c r="W10" t="s">
-        <v>40</v>
-      </c>
-      <c r="X10" t="s">
-        <v>40</v>
-      </c>
-      <c r="Y10" t="n">
+      <c r="BR10" t="s">
+        <v>89</v>
+      </c>
+      <c r="BS10" t="s">
+        <v>90</v>
+      </c>
+      <c r="BT10" t="s">
+        <v>90</v>
+      </c>
+      <c r="BU10" t="n">
         <v>11</v>
       </c>
-      <c r="Z10" t="n">
+      <c r="BV10" t="n">
         <v>9</v>
       </c>
-      <c r="AA10" t="n">
+      <c r="BW10" t="n">
         <v>1.15</v>
       </c>
-      <c r="AB10" t="n">
+      <c r="BX10" t="n">
         <v>1.15</v>
       </c>
-      <c r="AC10" t="n">
+      <c r="BY10" t="n">
         <v>1.15</v>
       </c>
-      <c r="AD10" t="n">
+      <c r="BZ10" t="n">
         <v>1.15</v>
       </c>
-      <c r="AE10" t="s">
-        <v>41</v>
-      </c>
-      <c r="AF10" t="s">
-        <v>41</v>
-      </c>
-      <c r="AG10" t="s">
-        <v>41</v>
-      </c>
-      <c r="AH10" t="s">
-        <v>42</v>
+      <c r="CA10" t="s">
+        <v>91</v>
+      </c>
+      <c r="CB10" t="s">
+        <v>91</v>
+      </c>
+      <c r="CC10" t="s">
+        <v>91</v>
+      </c>
+      <c r="CD10" t="s">
+        <v>92</v>
       </c>
     </row>
     <row r="11">
@@ -1603,31 +3241,31 @@
       </c>
       <c r="B11"/>
       <c r="C11" t="s">
-        <v>55</v>
+        <v>105</v>
       </c>
       <c r="D11" t="s">
-        <v>59</v>
+        <v>109</v>
       </c>
       <c r="E11" t="s">
-        <v>57</v>
+        <v>107</v>
       </c>
       <c r="F11" t="s">
-        <v>52</v>
+        <v>102</v>
       </c>
       <c r="G11" t="n">
         <v>200</v>
       </c>
       <c r="H11" t="n">
-        <v>215.8</v>
+        <v>210.3</v>
       </c>
       <c r="I11" t="n">
-        <v>415.8</v>
+        <v>410.2</v>
       </c>
       <c r="J11" t="n">
         <v>19.2</v>
       </c>
       <c r="K11" t="n">
-        <v>20.8</v>
+        <v>20.7</v>
       </c>
       <c r="L11" t="n">
         <v>39.9</v>
@@ -1636,67 +3274,211 @@
         <v>12.5</v>
       </c>
       <c r="N11" t="n">
-        <v>15.8</v>
+        <v>15.7</v>
       </c>
       <c r="O11" t="n">
         <v>28.2</v>
       </c>
       <c r="P11" t="n">
+        <v>68</v>
+      </c>
+      <c r="Q11" t="n">
+        <v>410.2</v>
+      </c>
+      <c r="R11" t="n">
+        <v>39.9</v>
+      </c>
+      <c r="S11" t="n">
+        <v>28.2</v>
+      </c>
+      <c r="T11" t="n">
+        <v>68</v>
+      </c>
+      <c r="U11" t="n">
+        <v>201.2</v>
+      </c>
+      <c r="V11" t="n">
+        <v>203.4</v>
+      </c>
+      <c r="W11" t="n">
+        <v>404.6</v>
+      </c>
+      <c r="X11" t="n">
+        <v>18.6</v>
+      </c>
+      <c r="Y11" t="n">
+        <v>21.2</v>
+      </c>
+      <c r="Z11" t="n">
+        <v>39.8</v>
+      </c>
+      <c r="AA11" t="n">
+        <v>12.9</v>
+      </c>
+      <c r="AB11" t="n">
+        <v>15.1</v>
+      </c>
+      <c r="AC11" t="n">
+        <v>28</v>
+      </c>
+      <c r="AD11" t="n">
+        <v>67.9</v>
+      </c>
+      <c r="AE11" t="n">
+        <v>202</v>
+      </c>
+      <c r="AF11" t="n">
+        <v>119</v>
+      </c>
+      <c r="AG11" t="n">
+        <v>1</v>
+      </c>
+      <c r="AH11" t="s">
+        <v>88</v>
+      </c>
+      <c r="AI11" t="n">
+        <v>336.2</v>
+      </c>
+      <c r="AJ11" t="n">
+        <v>36.2</v>
+      </c>
+      <c r="AK11" t="n">
+        <v>25.5</v>
+      </c>
+      <c r="AL11" t="n">
+        <v>61.7</v>
+      </c>
+      <c r="AM11" t="n">
+        <v>68.1</v>
+      </c>
+      <c r="AN11" t="n">
+        <v>73.6</v>
+      </c>
+      <c r="AO11" t="n">
+        <v>198.7</v>
+      </c>
+      <c r="AP11" t="n">
+        <v>217.2</v>
+      </c>
+      <c r="AQ11" t="n">
+        <v>415.9</v>
+      </c>
+      <c r="AR11" t="n">
+        <v>19.7</v>
+      </c>
+      <c r="AS11" t="n">
+        <v>20.2</v>
+      </c>
+      <c r="AT11" t="n">
+        <v>39.9</v>
+      </c>
+      <c r="AU11" t="n">
+        <v>12</v>
+      </c>
+      <c r="AV11" t="n">
+        <v>16.3</v>
+      </c>
+      <c r="AW11" t="n">
+        <v>28.3</v>
+      </c>
+      <c r="AX11" t="n">
         <v>68.2</v>
       </c>
-      <c r="Q11" t="s">
-        <v>59</v>
-      </c>
-      <c r="R11" t="n">
+      <c r="AY11" t="n">
+        <v>218</v>
+      </c>
+      <c r="AZ11" t="n">
+        <v>120</v>
+      </c>
+      <c r="BA11" t="n">
+        <v>0</v>
+      </c>
+      <c r="BB11" t="s">
+        <v>87</v>
+      </c>
+      <c r="BC11" t="n">
+        <v>380.9</v>
+      </c>
+      <c r="BD11" t="n">
+        <v>36.6</v>
+      </c>
+      <c r="BE11" t="n">
+        <v>25.7</v>
+      </c>
+      <c r="BF11" t="n">
+        <v>62.3</v>
+      </c>
+      <c r="BG11" t="n">
+        <v>68.2</v>
+      </c>
+      <c r="BH11" t="n">
+        <v>74.1</v>
+      </c>
+      <c r="BI11" t="n">
+        <v>11.3</v>
+      </c>
+      <c r="BJ11" t="n">
+        <v>0</v>
+      </c>
+      <c r="BK11" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="BL11" t="n">
+        <v>0.4</v>
+      </c>
+      <c r="BM11" t="s">
+        <v>109</v>
+      </c>
+      <c r="BN11" t="n">
         <v>6</v>
       </c>
-      <c r="S11" t="n">
+      <c r="BO11" t="n">
         <v>1.117</v>
       </c>
-      <c r="T11" t="n">
+      <c r="BP11" t="n">
         <v>1.121</v>
       </c>
-      <c r="U11" t="n">
+      <c r="BQ11" t="n">
         <v>1.321</v>
       </c>
-      <c r="V11" t="s">
-        <v>39</v>
-      </c>
-      <c r="W11" t="s">
-        <v>40</v>
-      </c>
-      <c r="X11" t="s">
-        <v>40</v>
-      </c>
-      <c r="Y11" t="n">
+      <c r="BR11" t="s">
+        <v>89</v>
+      </c>
+      <c r="BS11" t="s">
+        <v>90</v>
+      </c>
+      <c r="BT11" t="s">
+        <v>90</v>
+      </c>
+      <c r="BU11" t="n">
         <v>11</v>
       </c>
-      <c r="Z11" t="n">
+      <c r="BV11" t="n">
         <v>9</v>
       </c>
-      <c r="AA11" t="n">
+      <c r="BW11" t="n">
         <v>1.15</v>
       </c>
-      <c r="AB11" t="n">
+      <c r="BX11" t="n">
         <v>1.15</v>
       </c>
-      <c r="AC11" t="n">
+      <c r="BY11" t="n">
         <v>1.15</v>
       </c>
-      <c r="AD11" t="n">
+      <c r="BZ11" t="n">
         <v>1.15</v>
       </c>
-      <c r="AE11" t="s">
-        <v>41</v>
-      </c>
-      <c r="AF11" t="s">
-        <v>41</v>
-      </c>
-      <c r="AG11" t="s">
-        <v>41</v>
-      </c>
-      <c r="AH11" t="s">
-        <v>42</v>
+      <c r="CA11" t="s">
+        <v>91</v>
+      </c>
+      <c r="CB11" t="s">
+        <v>91</v>
+      </c>
+      <c r="CC11" t="s">
+        <v>91</v>
+      </c>
+      <c r="CD11" t="s">
+        <v>92</v>
       </c>
     </row>
     <row r="12">
@@ -1705,34 +3487,34 @@
       </c>
       <c r="B12"/>
       <c r="C12" t="s">
-        <v>55</v>
+        <v>105</v>
       </c>
       <c r="D12" t="s">
-        <v>60</v>
+        <v>110</v>
       </c>
       <c r="E12" t="s">
-        <v>57</v>
+        <v>107</v>
       </c>
       <c r="F12" t="s">
-        <v>52</v>
+        <v>102</v>
       </c>
       <c r="G12" t="n">
         <v>202</v>
       </c>
       <c r="H12" t="n">
-        <v>218</v>
+        <v>212.4</v>
       </c>
       <c r="I12" t="n">
-        <v>419.9</v>
+        <v>414.4</v>
       </c>
       <c r="J12" t="n">
         <v>18.9</v>
       </c>
       <c r="K12" t="n">
-        <v>20.5</v>
+        <v>20.4</v>
       </c>
       <c r="L12" t="n">
-        <v>39.4</v>
+        <v>39.3</v>
       </c>
       <c r="M12" t="n">
         <v>12.7</v>
@@ -1744,61 +3526,205 @@
         <v>28.8</v>
       </c>
       <c r="P12" t="n">
-        <v>68.2</v>
-      </c>
-      <c r="Q12" t="s">
-        <v>60</v>
+        <v>68.1</v>
+      </c>
+      <c r="Q12" t="n">
+        <v>414.4</v>
       </c>
       <c r="R12" t="n">
+        <v>39.3</v>
+      </c>
+      <c r="S12" t="n">
+        <v>28.8</v>
+      </c>
+      <c r="T12" t="n">
+        <v>68.1</v>
+      </c>
+      <c r="U12" t="n">
+        <v>203.2</v>
+      </c>
+      <c r="V12" t="n">
+        <v>205.5</v>
+      </c>
+      <c r="W12" t="n">
+        <v>408.7</v>
+      </c>
+      <c r="X12" t="n">
+        <v>18.4</v>
+      </c>
+      <c r="Y12" t="n">
+        <v>20.9</v>
+      </c>
+      <c r="Z12" t="n">
+        <v>39.3</v>
+      </c>
+      <c r="AA12" t="n">
+        <v>13.2</v>
+      </c>
+      <c r="AB12" t="n">
+        <v>15.4</v>
+      </c>
+      <c r="AC12" t="n">
+        <v>28.6</v>
+      </c>
+      <c r="AD12" t="n">
+        <v>67.9</v>
+      </c>
+      <c r="AE12" t="n">
+        <v>204</v>
+      </c>
+      <c r="AF12" t="n">
+        <v>119</v>
+      </c>
+      <c r="AG12" t="n">
+        <v>1</v>
+      </c>
+      <c r="AH12" t="s">
+        <v>88</v>
+      </c>
+      <c r="AI12" t="n">
+        <v>340.2</v>
+      </c>
+      <c r="AJ12" t="n">
+        <v>35.7</v>
+      </c>
+      <c r="AK12" t="n">
+        <v>26.1</v>
+      </c>
+      <c r="AL12" t="n">
+        <v>61.8</v>
+      </c>
+      <c r="AM12" t="n">
+        <v>68.1</v>
+      </c>
+      <c r="AN12" t="n">
+        <v>73.6</v>
+      </c>
+      <c r="AO12" t="n">
+        <v>200.7</v>
+      </c>
+      <c r="AP12" t="n">
+        <v>219.3</v>
+      </c>
+      <c r="AQ12" t="n">
+        <v>420</v>
+      </c>
+      <c r="AR12" t="n">
+        <v>19.5</v>
+      </c>
+      <c r="AS12" t="n">
+        <v>19.9</v>
+      </c>
+      <c r="AT12" t="n">
+        <v>39.3</v>
+      </c>
+      <c r="AU12" t="n">
+        <v>12.3</v>
+      </c>
+      <c r="AV12" t="n">
+        <v>16.7</v>
+      </c>
+      <c r="AW12" t="n">
+        <v>28.9</v>
+      </c>
+      <c r="AX12" t="n">
+        <v>68.3</v>
+      </c>
+      <c r="AY12" t="n">
+        <v>220</v>
+      </c>
+      <c r="AZ12" t="n">
+        <v>120</v>
+      </c>
+      <c r="BA12" t="n">
+        <v>0</v>
+      </c>
+      <c r="BB12" t="s">
+        <v>87</v>
+      </c>
+      <c r="BC12" t="n">
+        <v>385</v>
+      </c>
+      <c r="BD12" t="n">
+        <v>36.2</v>
+      </c>
+      <c r="BE12" t="n">
+        <v>26.3</v>
+      </c>
+      <c r="BF12" t="n">
+        <v>62.5</v>
+      </c>
+      <c r="BG12" t="n">
+        <v>68.3</v>
+      </c>
+      <c r="BH12" t="n">
+        <v>74.1</v>
+      </c>
+      <c r="BI12" t="n">
+        <v>11.4</v>
+      </c>
+      <c r="BJ12" t="n">
+        <v>0</v>
+      </c>
+      <c r="BK12" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="BL12" t="n">
+        <v>0.4</v>
+      </c>
+      <c r="BM12" t="s">
+        <v>110</v>
+      </c>
+      <c r="BN12" t="n">
         <v>8</v>
       </c>
-      <c r="S12" t="n">
+      <c r="BO12" t="n">
         <v>1.129</v>
       </c>
-      <c r="T12" t="n">
+      <c r="BP12" t="n">
         <v>1.105</v>
       </c>
-      <c r="U12" t="n">
+      <c r="BQ12" t="n">
         <v>1.35</v>
       </c>
-      <c r="V12" t="s">
-        <v>39</v>
-      </c>
-      <c r="W12" t="s">
-        <v>40</v>
-      </c>
-      <c r="X12" t="s">
-        <v>40</v>
-      </c>
-      <c r="Y12" t="n">
+      <c r="BR12" t="s">
+        <v>89</v>
+      </c>
+      <c r="BS12" t="s">
+        <v>90</v>
+      </c>
+      <c r="BT12" t="s">
+        <v>90</v>
+      </c>
+      <c r="BU12" t="n">
         <v>11</v>
       </c>
-      <c r="Z12" t="n">
+      <c r="BV12" t="n">
         <v>9</v>
       </c>
-      <c r="AA12" t="n">
+      <c r="BW12" t="n">
         <v>1.15</v>
       </c>
-      <c r="AB12" t="n">
+      <c r="BX12" t="n">
         <v>1.15</v>
       </c>
-      <c r="AC12" t="n">
+      <c r="BY12" t="n">
         <v>1.15</v>
       </c>
-      <c r="AD12" t="n">
+      <c r="BZ12" t="n">
         <v>1.15</v>
       </c>
-      <c r="AE12" t="s">
-        <v>41</v>
-      </c>
-      <c r="AF12" t="s">
-        <v>41</v>
-      </c>
-      <c r="AG12" t="s">
-        <v>41</v>
-      </c>
-      <c r="AH12" t="s">
-        <v>42</v>
+      <c r="CA12" t="s">
+        <v>91</v>
+      </c>
+      <c r="CB12" t="s">
+        <v>91</v>
+      </c>
+      <c r="CC12" t="s">
+        <v>91</v>
+      </c>
+      <c r="CD12" t="s">
+        <v>92</v>
       </c>
     </row>
     <row r="13">
@@ -1807,100 +3733,244 @@
       </c>
       <c r="B13"/>
       <c r="C13" t="s">
-        <v>55</v>
+        <v>105</v>
       </c>
       <c r="D13" t="s">
-        <v>61</v>
+        <v>111</v>
       </c>
       <c r="E13" t="s">
-        <v>57</v>
+        <v>107</v>
       </c>
       <c r="F13" t="s">
-        <v>52</v>
+        <v>102</v>
       </c>
       <c r="G13" t="n">
         <v>195.4</v>
       </c>
       <c r="H13" t="n">
-        <v>210.9</v>
+        <v>205.3</v>
       </c>
       <c r="I13" t="n">
-        <v>406.2</v>
+        <v>400.7</v>
       </c>
       <c r="J13" t="n">
         <v>19.7</v>
       </c>
       <c r="K13" t="n">
-        <v>21.3</v>
+        <v>21.2</v>
       </c>
       <c r="L13" t="n">
-        <v>41.1</v>
+        <v>40.9</v>
       </c>
       <c r="M13" t="n">
         <v>10.3</v>
       </c>
       <c r="N13" t="n">
-        <v>13.1</v>
+        <v>13</v>
       </c>
       <c r="O13" t="n">
-        <v>23.4</v>
+        <v>23.3</v>
       </c>
       <c r="P13" t="n">
+        <v>64.3</v>
+      </c>
+      <c r="Q13" t="n">
+        <v>400.7</v>
+      </c>
+      <c r="R13" t="n">
+        <v>40.9</v>
+      </c>
+      <c r="S13" t="n">
+        <v>23.3</v>
+      </c>
+      <c r="T13" t="n">
+        <v>64.3</v>
+      </c>
+      <c r="U13" t="n">
+        <v>196.6</v>
+      </c>
+      <c r="V13" t="n">
+        <v>198.4</v>
+      </c>
+      <c r="W13" t="n">
+        <v>395</v>
+      </c>
+      <c r="X13" t="n">
+        <v>19.1</v>
+      </c>
+      <c r="Y13" t="n">
+        <v>21.7</v>
+      </c>
+      <c r="Z13" t="n">
+        <v>40.9</v>
+      </c>
+      <c r="AA13" t="n">
+        <v>10.7</v>
+      </c>
+      <c r="AB13" t="n">
+        <v>12.5</v>
+      </c>
+      <c r="AC13" t="n">
+        <v>23.2</v>
+      </c>
+      <c r="AD13" t="n">
+        <v>64</v>
+      </c>
+      <c r="AE13" t="n">
+        <v>197</v>
+      </c>
+      <c r="AF13" t="n">
+        <v>119</v>
+      </c>
+      <c r="AG13" t="n">
+        <v>1</v>
+      </c>
+      <c r="AH13" t="s">
+        <v>88</v>
+      </c>
+      <c r="AI13" t="n">
+        <v>326.6</v>
+      </c>
+      <c r="AJ13" t="n">
+        <v>36.8</v>
+      </c>
+      <c r="AK13" t="n">
+        <v>20.9</v>
+      </c>
+      <c r="AL13" t="n">
+        <v>57.7</v>
+      </c>
+      <c r="AM13" t="n">
+        <v>64.4</v>
+      </c>
+      <c r="AN13" t="n">
+        <v>69.7</v>
+      </c>
+      <c r="AO13" t="n">
+        <v>194.2</v>
+      </c>
+      <c r="AP13" t="n">
+        <v>212.2</v>
+      </c>
+      <c r="AQ13" t="n">
+        <v>406.3</v>
+      </c>
+      <c r="AR13" t="n">
+        <v>20.3</v>
+      </c>
+      <c r="AS13" t="n">
+        <v>20.7</v>
+      </c>
+      <c r="AT13" t="n">
+        <v>41</v>
+      </c>
+      <c r="AU13" t="n">
+        <v>10</v>
+      </c>
+      <c r="AV13" t="n">
+        <v>13.5</v>
+      </c>
+      <c r="AW13" t="n">
+        <v>23.5</v>
+      </c>
+      <c r="AX13" t="n">
         <v>64.5</v>
       </c>
-      <c r="Q13" t="s">
-        <v>62</v>
-      </c>
-      <c r="R13" t="n">
+      <c r="AY13" t="n">
+        <v>213</v>
+      </c>
+      <c r="AZ13" t="n">
+        <v>120</v>
+      </c>
+      <c r="BA13" t="n">
+        <v>0</v>
+      </c>
+      <c r="BB13" t="s">
+        <v>87</v>
+      </c>
+      <c r="BC13" t="n">
+        <v>371.3</v>
+      </c>
+      <c r="BD13" t="n">
+        <v>37.6</v>
+      </c>
+      <c r="BE13" t="n">
+        <v>21.3</v>
+      </c>
+      <c r="BF13" t="n">
+        <v>58.8</v>
+      </c>
+      <c r="BG13" t="n">
+        <v>64.5</v>
+      </c>
+      <c r="BH13" t="n">
+        <v>70.2</v>
+      </c>
+      <c r="BI13" t="n">
+        <v>11.3</v>
+      </c>
+      <c r="BJ13" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="BK13" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="BL13" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="BM13" t="s">
+        <v>112</v>
+      </c>
+      <c r="BN13" t="n">
         <v>10</v>
       </c>
-      <c r="S13" t="n">
+      <c r="BO13" t="n">
         <v>1.092</v>
       </c>
-      <c r="T13" t="n">
+      <c r="BP13" t="n">
         <v>1.152</v>
       </c>
-      <c r="U13" t="n">
+      <c r="BQ13" t="n">
         <v>1.096</v>
       </c>
-      <c r="V13" t="s">
-        <v>39</v>
-      </c>
-      <c r="W13" t="s">
-        <v>40</v>
-      </c>
-      <c r="X13" t="s">
-        <v>40</v>
-      </c>
-      <c r="Y13" t="n">
+      <c r="BR13" t="s">
+        <v>89</v>
+      </c>
+      <c r="BS13" t="s">
+        <v>90</v>
+      </c>
+      <c r="BT13" t="s">
+        <v>90</v>
+      </c>
+      <c r="BU13" t="n">
         <v>11</v>
       </c>
-      <c r="Z13" t="n">
+      <c r="BV13" t="n">
         <v>9</v>
       </c>
-      <c r="AA13" t="n">
+      <c r="BW13" t="n">
         <v>1.15</v>
       </c>
-      <c r="AB13" t="n">
+      <c r="BX13" t="n">
         <v>1.15</v>
       </c>
-      <c r="AC13" t="n">
+      <c r="BY13" t="n">
         <v>1.15</v>
       </c>
-      <c r="AD13" t="n">
+      <c r="BZ13" t="n">
         <v>1.15</v>
       </c>
-      <c r="AE13" t="s">
-        <v>41</v>
-      </c>
-      <c r="AF13" t="s">
-        <v>41</v>
-      </c>
-      <c r="AG13" t="s">
-        <v>41</v>
-      </c>
-      <c r="AH13" t="s">
-        <v>42</v>
+      <c r="CA13" t="s">
+        <v>91</v>
+      </c>
+      <c r="CB13" t="s">
+        <v>91</v>
+      </c>
+      <c r="CC13" t="s">
+        <v>91</v>
+      </c>
+      <c r="CD13" t="s">
+        <v>92</v>
       </c>
     </row>
   </sheetData>

</xml_diff>